<commit_message>
Update Alex Lodise (Low-A, Augusta GreenJackets) and Cam Leiter (Low-A, Ontario Tower Buzzers)
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -1973,12 +1973,12 @@
       </c>
       <c r="D19" s="112" t="inlineStr">
         <is>
-          <t>High-A</t>
+          <t>Low-A</t>
         </is>
       </c>
       <c r="E19" s="113" t="inlineStr">
         <is>
-          <t>Rome Emperors</t>
+          <t>Augusta GreenJackets</t>
         </is>
       </c>
       <c r="F19" s="112" t="n">
@@ -2575,12 +2575,12 @@
       </c>
       <c r="D33" s="136" t="inlineStr">
         <is>
-          <t>Rookie</t>
+          <t>Low-A</t>
         </is>
       </c>
       <c r="E33" s="137" t="inlineStr">
         <is>
-          <t>ACL/AZL</t>
+          <t>Ontario Tower Buzzers</t>
         </is>
       </c>
       <c r="F33" s="136" t="n">

</xml_diff>

<commit_message>
Roster corrections: Tibbs->OKC Comets, Dinges->Wisconsin Timber Rattlers, Lodise->Low-A Augusta, Leiter->Low-A Ontario
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="E10" s="93" t="inlineStr">
         <is>
-          <t>Oklahoma City Baseball Club</t>
+          <t>Oklahoma City Comets</t>
         </is>
       </c>
       <c r="F10" s="92" t="n">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="E20" s="117" t="inlineStr">
         <is>
-          <t>Carolina Mudcats</t>
+          <t>Wisconsin Timber Rattlers</t>
         </is>
       </c>
       <c r="F20" s="116" t="n">

</xml_diff>

<commit_message>
Roster updates: Faurot/Volini->High-A Beloit, West->Low-A Dunedin, Vincent->AAA El Paso, Montgomery->Low-A Fort Wayne, Whittaker/Tejeda->High-A, Williams->Low-A Jupiter
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -2231,12 +2231,12 @@
       </c>
       <c r="D25" s="124" t="inlineStr">
         <is>
-          <t>Low-A</t>
+          <t>High-A</t>
         </is>
       </c>
       <c r="E25" s="125" t="inlineStr">
         <is>
-          <t>Fredericksburg Nationals</t>
+          <t>Wilmington Blue Rocks</t>
         </is>
       </c>
       <c r="F25" s="124" t="n">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="D26" s="120" t="inlineStr">
         <is>
-          <t>Low-A</t>
+          <t>High-A</t>
         </is>
       </c>
       <c r="E26" s="121" t="inlineStr">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="E28" s="121" t="inlineStr">
         <is>
-          <t>Lake Elsinore Storm</t>
+          <t>Fort Wayne TinCaps</t>
         </is>
       </c>
       <c r="F28" s="120" t="n">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="D29" s="128" t="inlineStr">
         <is>
-          <t>Low-A</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="E29" s="129" t="inlineStr">
         <is>
-          <t>Lake Elsinore Storm</t>
+          <t>El Paso Chihuahuas</t>
         </is>
       </c>
       <c r="F29" s="128" t="n">
@@ -2449,12 +2449,12 @@
       </c>
       <c r="D30" s="132" t="inlineStr">
         <is>
-          <t>Rookie</t>
+          <t>Low-A</t>
         </is>
       </c>
       <c r="E30" s="133" t="inlineStr">
         <is>
-          <t>FCL/Jupiter</t>
+          <t>Jupiter Hammerheads</t>
         </is>
       </c>
       <c r="F30" s="132" t="n">
@@ -2491,12 +2491,12 @@
       </c>
       <c r="D31" s="136" t="inlineStr">
         <is>
-          <t>Rookie</t>
+          <t>High-A</t>
         </is>
       </c>
       <c r="E31" s="137" t="inlineStr">
         <is>
-          <t>FCL/Jupiter</t>
+          <t>Beloit Sky Carp</t>
         </is>
       </c>
       <c r="F31" s="136" t="n">
@@ -2533,12 +2533,12 @@
       </c>
       <c r="D32" s="132" t="inlineStr">
         <is>
-          <t>Rookie</t>
+          <t>High-A</t>
         </is>
       </c>
       <c r="E32" s="133" t="inlineStr">
         <is>
-          <t>FCL/Jupiter</t>
+          <t>Beloit Sky Carp</t>
         </is>
       </c>
       <c r="F32" s="132" t="n">
@@ -2745,12 +2745,12 @@
       </c>
       <c r="D37" s="136" t="inlineStr">
         <is>
-          <t>Rookie</t>
+          <t>Low-A</t>
         </is>
       </c>
       <c r="E37" s="137" t="inlineStr">
         <is>
-          <t>ACL/AZL</t>
+          <t>Dunedin Blue Jays</t>
         </is>
       </c>
       <c r="F37" s="136" t="n">

</xml_diff>

<commit_message>
Roster update: Gage Harrelson -> High-A / Tri-City Dust Devils (Angels)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -2703,12 +2703,12 @@
       </c>
       <c r="D36" s="132" t="inlineStr">
         <is>
-          <t>Rookie</t>
+          <t>High-A</t>
         </is>
       </c>
       <c r="E36" s="133" t="inlineStr">
         <is>
-          <t>ACL Angels</t>
+          <t>Tri-City Dust Devils</t>
         </is>
       </c>
       <c r="F36" s="132" t="n">

</xml_diff>

<commit_message>
Stats refresh: regenerate dashboard with Apr 6 2026 stats
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -3273,57 +3273,57 @@
       </c>
       <c r="E3" s="168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="168" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" s="168" t="inlineStr">
         <is>
-          <t>.132</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L3" s="168" t="inlineStr">
         <is>
-          <t>.233</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" s="168" t="inlineStr">
         <is>
-          <t>.184</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" s="168" t="inlineStr">
         <is>
-          <t>.417</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -3350,57 +3350,57 @@
       </c>
       <c r="E4" s="168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="168" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="168" t="inlineStr">
         <is>
-          <t>.273</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="168" t="inlineStr">
         <is>
-          <t>.400</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" s="168" t="inlineStr">
         <is>
-          <t>.485</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="168" t="inlineStr">
         <is>
-          <t>.885</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -3504,57 +3504,57 @@
       </c>
       <c r="E6" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="168" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="168" t="inlineStr">
         <is>
-          <t>.474</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="168" t="inlineStr">
         <is>
-          <t>.535</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" s="168" t="inlineStr">
         <is>
-          <t>1.184</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" s="168" t="inlineStr">
         <is>
-          <t>1.719</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -3735,57 +3735,57 @@
       </c>
       <c r="E9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="168" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M9" s="168" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N9" s="168" t="inlineStr">
         <is>
-          <t>2.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -3812,57 +3812,57 @@
       </c>
       <c r="E10" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="168" t="inlineStr">
         <is>
-          <t>.538</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="168" t="inlineStr">
         <is>
-          <t>.993</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -3966,57 +3966,57 @@
       </c>
       <c r="E12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4043,57 +4043,57 @@
       </c>
       <c r="E13" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4120,57 +4120,57 @@
       </c>
       <c r="E14" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="168" t="inlineStr">
         <is>
-          <t>.385</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J14" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L14" s="168" t="inlineStr">
         <is>
-          <t>.429</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M14" s="168" t="inlineStr">
         <is>
-          <t>.462</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N14" s="168" t="inlineStr">
         <is>
-          <t>.891</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4351,57 +4351,57 @@
       </c>
       <c r="E17" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N17" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4666,57 +4666,57 @@
       </c>
       <c r="E23" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="168" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="168" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4743,57 +4743,57 @@
       </c>
       <c r="E24" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K24" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L24" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M24" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N24" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4820,57 +4820,57 @@
       </c>
       <c r="E25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="168" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="168" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="168" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N25" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4897,57 +4897,57 @@
       </c>
       <c r="E26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="168" t="inlineStr">
         <is>
-          <t>2.45</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -4974,57 +4974,57 @@
       </c>
       <c r="E27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" s="168" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K27" s="168" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L27" s="168" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M27" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N27" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5051,57 +5051,57 @@
       </c>
       <c r="E28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="168" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="168" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="168" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M28" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5128,57 +5128,57 @@
       </c>
       <c r="E29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J29" s="168" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K29" s="168" t="inlineStr">
         <is>
-          <t>10.57</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L29" s="168" t="inlineStr">
         <is>
-          <t>2.48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M29" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N29" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5282,57 +5282,57 @@
       </c>
       <c r="E31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="168" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="168" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="168" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N31" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -6052,57 +6052,57 @@
       </c>
       <c r="E41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" s="168" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K41" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L41" s="168" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M41" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 11:38</t>
+          <t>04/06/2026 13:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add modal player cards: click any card to see full stats, bio, and MiLB link
- Replaced flat card design with portrait-style card + 4-stat strip (AVG/HR/OPS/G or ERA/WHIP/K/G)
- Added modal overlay on card click: shows headshot, org, team, draft info, notes, full stats table, and MiLB link
- Updated read_roster() to pull draft year/round/pick and notes from xlsx
- No external links on card click — everything in-page

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -3323,7 +3323,7 @@
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4093,7 +4093,7 @@
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4870,7 +4870,7 @@
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -6102,7 +6102,7 @@
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:42</t>
+          <t>04/06/2026 13:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix modal cards: correct f-string/JSON conflict, wire up onclick handlers
The modal JSON data was silently dropped because JSON curly braces
conflicted with Python f-string syntax. Fixed by using a placeholder
string replaced post-render. Cards now have working onclick="openModal(idx)"
and MODAL_DATA is correctly embedded in the page.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -3323,7 +3323,7 @@
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4093,7 +4093,7 @@
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4870,7 +4870,7 @@
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -6102,7 +6102,7 @@
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/06/2026 13:55</t>
+          <t>04/06/2026 14:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add modal player cards with stats — fix live site click behavior
- noles_stats_updater.py: New portrait card design with onclick openModal()
- Added card stat strip (4 stats: AVG/HR/OPS/G or ERA/WHIP/K/G)
- Added modal overlay with full stats table, headshot, draft info, notes
- MODAL_DATA JSON injected post-render to avoid f-string brace conflicts
- index.html updated to match dashboard (fixes homepage not updating)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -3273,57 +3273,57 @@
       </c>
       <c r="E3" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="168" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" s="168" t="inlineStr">
         <is>
-          <t>.146</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L3" s="168" t="inlineStr">
         <is>
-          <t>.255</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" s="168" t="inlineStr">
         <is>
-          <t>.268</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" s="168" t="inlineStr">
         <is>
-          <t>.523</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -3350,57 +3350,57 @@
       </c>
       <c r="E4" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="168" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="168" t="inlineStr">
         <is>
-          <t>.297</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="168" t="inlineStr">
         <is>
-          <t>.422</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" s="168" t="inlineStr">
         <is>
-          <t>.595</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="168" t="inlineStr">
         <is>
-          <t>1.017</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -3427,57 +3427,57 @@
       </c>
       <c r="E5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" s="168" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -3504,57 +3504,57 @@
       </c>
       <c r="E6" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="168" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="168" t="inlineStr">
         <is>
-          <t>.474</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="168" t="inlineStr">
         <is>
-          <t>.535</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" s="168" t="inlineStr">
         <is>
-          <t>1.184</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" s="168" t="inlineStr">
         <is>
-          <t>1.719</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -3735,57 +3735,57 @@
       </c>
       <c r="E9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="168" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M9" s="168" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N9" s="168" t="inlineStr">
         <is>
-          <t>2.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -3812,57 +3812,57 @@
       </c>
       <c r="E10" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="168" t="inlineStr">
         <is>
-          <t>.538</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="168" t="inlineStr">
         <is>
-          <t>.993</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -3966,57 +3966,57 @@
       </c>
       <c r="E12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4043,57 +4043,57 @@
       </c>
       <c r="E13" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4120,57 +4120,57 @@
       </c>
       <c r="E14" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="168" t="inlineStr">
         <is>
-          <t>.385</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J14" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L14" s="168" t="inlineStr">
         <is>
-          <t>.429</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M14" s="168" t="inlineStr">
         <is>
-          <t>.462</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N14" s="168" t="inlineStr">
         <is>
-          <t>.891</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4351,57 +4351,57 @@
       </c>
       <c r="E17" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N17" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4666,57 +4666,57 @@
       </c>
       <c r="E23" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="168" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="168" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4743,57 +4743,57 @@
       </c>
       <c r="E24" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K24" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L24" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M24" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N24" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4820,57 +4820,57 @@
       </c>
       <c r="E25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="168" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="168" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="168" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N25" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4897,57 +4897,57 @@
       </c>
       <c r="E26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="168" t="inlineStr">
         <is>
-          <t>2.45</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -4974,57 +4974,57 @@
       </c>
       <c r="E27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" s="168" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K27" s="168" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L27" s="168" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M27" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N27" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5051,57 +5051,57 @@
       </c>
       <c r="E28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="168" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="168" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="168" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M28" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5128,57 +5128,57 @@
       </c>
       <c r="E29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J29" s="168" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K29" s="168" t="inlineStr">
         <is>
-          <t>10.57</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L29" s="168" t="inlineStr">
         <is>
-          <t>2.48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M29" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N29" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5282,57 +5282,57 @@
       </c>
       <c r="E31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="168" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="168" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="168" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N31" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -6052,57 +6052,57 @@
       </c>
       <c r="E41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" s="168" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K41" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L41" s="168" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M41" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:00</t>
+          <t>04/06/2026 14:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Force correct card layout into index.html and dashboard
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -3273,57 +3273,57 @@
       </c>
       <c r="E3" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="168" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" s="168" t="inlineStr">
         <is>
-          <t>.146</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L3" s="168" t="inlineStr">
         <is>
-          <t>.255</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" s="168" t="inlineStr">
         <is>
-          <t>.268</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" s="168" t="inlineStr">
         <is>
-          <t>.523</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -3350,57 +3350,57 @@
       </c>
       <c r="E4" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="168" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="168" t="inlineStr">
         <is>
-          <t>.297</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="168" t="inlineStr">
         <is>
-          <t>.422</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" s="168" t="inlineStr">
         <is>
-          <t>.595</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="168" t="inlineStr">
         <is>
-          <t>1.017</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -3427,57 +3427,57 @@
       </c>
       <c r="E5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" s="168" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -3504,57 +3504,57 @@
       </c>
       <c r="E6" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="168" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="168" t="inlineStr">
         <is>
-          <t>.474</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="168" t="inlineStr">
         <is>
-          <t>.535</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" s="168" t="inlineStr">
         <is>
-          <t>1.184</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" s="168" t="inlineStr">
         <is>
-          <t>1.719</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -3735,57 +3735,57 @@
       </c>
       <c r="E9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="168" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M9" s="168" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N9" s="168" t="inlineStr">
         <is>
-          <t>2.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -3812,57 +3812,57 @@
       </c>
       <c r="E10" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="168" t="inlineStr">
         <is>
-          <t>.538</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="168" t="inlineStr">
         <is>
-          <t>.993</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -3966,57 +3966,57 @@
       </c>
       <c r="E12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4043,57 +4043,57 @@
       </c>
       <c r="E13" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4120,57 +4120,57 @@
       </c>
       <c r="E14" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="168" t="inlineStr">
         <is>
-          <t>.385</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J14" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L14" s="168" t="inlineStr">
         <is>
-          <t>.429</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M14" s="168" t="inlineStr">
         <is>
-          <t>.462</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N14" s="168" t="inlineStr">
         <is>
-          <t>.891</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4351,57 +4351,57 @@
       </c>
       <c r="E17" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N17" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4666,57 +4666,57 @@
       </c>
       <c r="E23" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="168" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="168" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4743,57 +4743,57 @@
       </c>
       <c r="E24" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K24" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L24" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M24" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N24" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4820,57 +4820,57 @@
       </c>
       <c r="E25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="168" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="168" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="168" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N25" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4897,57 +4897,57 @@
       </c>
       <c r="E26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="168" t="inlineStr">
         <is>
-          <t>2.45</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -4974,57 +4974,57 @@
       </c>
       <c r="E27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" s="168" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K27" s="168" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L27" s="168" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M27" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N27" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5051,57 +5051,57 @@
       </c>
       <c r="E28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="168" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="168" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="168" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M28" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5128,57 +5128,57 @@
       </c>
       <c r="E29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J29" s="168" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K29" s="168" t="inlineStr">
         <is>
-          <t>10.57</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L29" s="168" t="inlineStr">
         <is>
-          <t>2.48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M29" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N29" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5282,57 +5282,57 @@
       </c>
       <c r="E31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="168" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="168" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="168" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N31" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -6052,57 +6052,57 @@
       </c>
       <c r="E41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" s="168" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K41" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L41" s="168" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M41" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 12:52</t>
+          <t>04/07/2026 06:44</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add IP/W/L/SV to pitcher card strip; batters already had G
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -3273,57 +3273,57 @@
       </c>
       <c r="E3" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="168" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" s="168" t="inlineStr">
         <is>
-          <t>.146</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L3" s="168" t="inlineStr">
         <is>
-          <t>.255</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" s="168" t="inlineStr">
         <is>
-          <t>.268</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" s="168" t="inlineStr">
         <is>
-          <t>.523</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -3350,57 +3350,57 @@
       </c>
       <c r="E4" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="168" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="168" t="inlineStr">
         <is>
-          <t>.297</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="168" t="inlineStr">
         <is>
-          <t>.422</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" s="168" t="inlineStr">
         <is>
-          <t>.595</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="168" t="inlineStr">
         <is>
-          <t>1.017</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -3427,57 +3427,57 @@
       </c>
       <c r="E5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" s="168" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -3504,57 +3504,57 @@
       </c>
       <c r="E6" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="168" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="168" t="inlineStr">
         <is>
-          <t>.474</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="168" t="inlineStr">
         <is>
-          <t>.535</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" s="168" t="inlineStr">
         <is>
-          <t>1.184</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" s="168" t="inlineStr">
         <is>
-          <t>1.719</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -3735,57 +3735,57 @@
       </c>
       <c r="E9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="168" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M9" s="168" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N9" s="168" t="inlineStr">
         <is>
-          <t>2.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -3812,57 +3812,57 @@
       </c>
       <c r="E10" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="168" t="inlineStr">
         <is>
-          <t>.538</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="168" t="inlineStr">
         <is>
-          <t>.993</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -3966,57 +3966,57 @@
       </c>
       <c r="E12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4043,57 +4043,57 @@
       </c>
       <c r="E13" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4120,57 +4120,57 @@
       </c>
       <c r="E14" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="168" t="inlineStr">
         <is>
-          <t>.385</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J14" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L14" s="168" t="inlineStr">
         <is>
-          <t>.429</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M14" s="168" t="inlineStr">
         <is>
-          <t>.462</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N14" s="168" t="inlineStr">
         <is>
-          <t>.891</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4351,57 +4351,57 @@
       </c>
       <c r="E17" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N17" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4666,57 +4666,57 @@
       </c>
       <c r="E23" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="168" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="168" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4743,57 +4743,57 @@
       </c>
       <c r="E24" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K24" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L24" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M24" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N24" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4820,57 +4820,57 @@
       </c>
       <c r="E25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="168" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="168" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="168" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N25" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4897,57 +4897,57 @@
       </c>
       <c r="E26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="168" t="inlineStr">
         <is>
-          <t>2.45</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -4974,57 +4974,57 @@
       </c>
       <c r="E27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" s="168" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K27" s="168" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L27" s="168" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M27" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N27" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5051,57 +5051,57 @@
       </c>
       <c r="E28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="168" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="168" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="168" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M28" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5128,57 +5128,57 @@
       </c>
       <c r="E29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J29" s="168" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K29" s="168" t="inlineStr">
         <is>
-          <t>10.57</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L29" s="168" t="inlineStr">
         <is>
-          <t>2.48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M29" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N29" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5282,57 +5282,57 @@
       </c>
       <c r="E31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="168" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="168" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="168" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N31" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -6052,57 +6052,57 @@
       </c>
       <c r="E41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" s="168" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K41" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L41" s="168" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M41" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 18:40</t>
+          <t>04/07/2026 10:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Garnet/gold initials placeholder for missing photos; fix modal photo wrap
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -3273,57 +3273,57 @@
       </c>
       <c r="E3" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="168" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" s="168" t="inlineStr">
         <is>
-          <t>.146</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L3" s="168" t="inlineStr">
         <is>
-          <t>.255</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" s="168" t="inlineStr">
         <is>
-          <t>.268</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" s="168" t="inlineStr">
         <is>
-          <t>.523</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -3350,57 +3350,57 @@
       </c>
       <c r="E4" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="168" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="168" t="inlineStr">
         <is>
-          <t>.297</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="168" t="inlineStr">
         <is>
-          <t>.422</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" s="168" t="inlineStr">
         <is>
-          <t>.595</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="168" t="inlineStr">
         <is>
-          <t>1.017</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -3427,57 +3427,57 @@
       </c>
       <c r="E5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" s="168" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -3504,57 +3504,57 @@
       </c>
       <c r="E6" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="168" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="168" t="inlineStr">
         <is>
-          <t>.474</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="168" t="inlineStr">
         <is>
-          <t>.535</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" s="168" t="inlineStr">
         <is>
-          <t>1.184</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" s="168" t="inlineStr">
         <is>
-          <t>1.719</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -3735,57 +3735,57 @@
       </c>
       <c r="E9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="168" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M9" s="168" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N9" s="168" t="inlineStr">
         <is>
-          <t>2.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -3812,57 +3812,57 @@
       </c>
       <c r="E10" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="168" t="inlineStr">
         <is>
-          <t>.538</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="168" t="inlineStr">
         <is>
-          <t>.993</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -3966,57 +3966,57 @@
       </c>
       <c r="E12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4043,57 +4043,57 @@
       </c>
       <c r="E13" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4120,57 +4120,57 @@
       </c>
       <c r="E14" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="168" t="inlineStr">
         <is>
-          <t>.385</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J14" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L14" s="168" t="inlineStr">
         <is>
-          <t>.429</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M14" s="168" t="inlineStr">
         <is>
-          <t>.462</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N14" s="168" t="inlineStr">
         <is>
-          <t>.891</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4351,57 +4351,57 @@
       </c>
       <c r="E17" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N17" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4666,57 +4666,57 @@
       </c>
       <c r="E23" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="168" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="168" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4743,57 +4743,57 @@
       </c>
       <c r="E24" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K24" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L24" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M24" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N24" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4820,57 +4820,57 @@
       </c>
       <c r="E25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="168" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="168" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="168" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N25" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4897,57 +4897,57 @@
       </c>
       <c r="E26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="168" t="inlineStr">
         <is>
-          <t>2.45</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -4974,57 +4974,57 @@
       </c>
       <c r="E27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" s="168" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K27" s="168" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L27" s="168" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M27" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N27" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5051,57 +5051,57 @@
       </c>
       <c r="E28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="168" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="168" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="168" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M28" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5128,57 +5128,57 @@
       </c>
       <c r="E29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J29" s="168" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K29" s="168" t="inlineStr">
         <is>
-          <t>10.57</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L29" s="168" t="inlineStr">
         <is>
-          <t>2.48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M29" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N29" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5282,57 +5282,57 @@
       </c>
       <c r="E31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="168" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="168" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="168" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N31" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -6052,57 +6052,57 @@
       </c>
       <c r="E41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" s="168" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K41" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L41" s="168" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M41" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 19:15</t>
+          <t>04/07/2026 13:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate with Shane at MLB
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -3273,57 +3273,57 @@
       </c>
       <c r="E3" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="168" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" s="168" t="inlineStr">
         <is>
-          <t>.146</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L3" s="168" t="inlineStr">
         <is>
-          <t>.255</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" s="168" t="inlineStr">
         <is>
-          <t>.268</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" s="168" t="inlineStr">
         <is>
-          <t>.523</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -3350,57 +3350,57 @@
       </c>
       <c r="E4" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="168" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="168" t="inlineStr">
         <is>
-          <t>.297</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="168" t="inlineStr">
         <is>
-          <t>.422</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" s="168" t="inlineStr">
         <is>
-          <t>.595</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="168" t="inlineStr">
         <is>
-          <t>1.017</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -3427,57 +3427,57 @@
       </c>
       <c r="E5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L5" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" s="168" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -3504,57 +3504,57 @@
       </c>
       <c r="E6" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="168" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="168" t="inlineStr">
         <is>
-          <t>.474</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="168" t="inlineStr">
         <is>
-          <t>.535</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" s="168" t="inlineStr">
         <is>
-          <t>1.184</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" s="168" t="inlineStr">
         <is>
-          <t>1.719</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -3735,57 +3735,57 @@
       </c>
       <c r="E9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="168" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="168" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M9" s="168" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N9" s="168" t="inlineStr">
         <is>
-          <t>2.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -3812,57 +3812,57 @@
       </c>
       <c r="E10" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="168" t="inlineStr">
         <is>
-          <t>.538</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="168" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="168" t="inlineStr">
         <is>
-          <t>.993</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -3966,57 +3966,57 @@
       </c>
       <c r="E12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="168" t="inlineStr">
         <is>
-          <t>.250</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4043,57 +4043,57 @@
       </c>
       <c r="E13" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M13" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4120,57 +4120,57 @@
       </c>
       <c r="E14" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="168" t="inlineStr">
         <is>
-          <t>.385</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J14" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L14" s="168" t="inlineStr">
         <is>
-          <t>.429</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M14" s="168" t="inlineStr">
         <is>
-          <t>.462</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N14" s="168" t="inlineStr">
         <is>
-          <t>.891</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4351,57 +4351,57 @@
       </c>
       <c r="E17" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N17" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4666,57 +4666,57 @@
       </c>
       <c r="E23" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="168" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="168" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4743,57 +4743,57 @@
       </c>
       <c r="E24" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K24" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L24" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M24" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N24" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4820,57 +4820,57 @@
       </c>
       <c r="E25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="168" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="168" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="168" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N25" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4897,57 +4897,57 @@
       </c>
       <c r="E26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="168" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="168" t="inlineStr">
         <is>
-          <t>2.45</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="168" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -4974,57 +4974,57 @@
       </c>
       <c r="E27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" s="168" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K27" s="168" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L27" s="168" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M27" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N27" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5051,57 +5051,57 @@
       </c>
       <c r="E28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="168" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="168" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="168" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M28" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5128,57 +5128,57 @@
       </c>
       <c r="E29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J29" s="168" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K29" s="168" t="inlineStr">
         <is>
-          <t>10.57</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L29" s="168" t="inlineStr">
         <is>
-          <t>2.48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M29" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N29" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5282,57 +5282,57 @@
       </c>
       <c r="E31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="168" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="168" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="168" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N31" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -6052,57 +6052,57 @@
       </c>
       <c r="E41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" s="168" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K41" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L41" s="168" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M41" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 20:25</t>
+          <t>04/07/2026 13:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Shane Drohan MLB/Brewers; regenerate with latest stats
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1547,12 +1547,12 @@
       </c>
       <c r="D9" s="88" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" s="89" t="inlineStr">
         <is>
-          <t>Nashville Sounds</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F9" s="88" t="n">
@@ -1567,7 +1567,7 @@
       <c r="I9" s="88" t="n"/>
       <c r="J9" s="90" t="inlineStr">
         <is>
-          <t>On 40-man roster; 2.27 ERA at Triple-A in 2025; called up to Boston Nov 2025, traded to MIL Feb 2026</t>
+          <t>Called up to MIL April 2026; traded from BOS to MIL Feb 2026</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4093,7 +4093,7 @@
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4870,7 +4870,7 @@
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -4964,12 +4964,12 @@
       </c>
       <c r="C27" s="168" t="inlineStr">
         <is>
-          <t>Nashville Sounds</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="D27" s="168" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E27" s="168" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -6102,7 +6102,7 @@
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/07/2026 13:27</t>
+          <t>04/07/2026 13:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add XML sitemap for Google Search Console
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$J$35</definedName>
@@ -3273,57 +3273,57 @@
       </c>
       <c r="E3" s="168" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="168" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" s="168" t="inlineStr">
         <is>
-          <t>.156</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K3" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L3" s="168" t="inlineStr">
         <is>
-          <t>.255</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" s="168" t="inlineStr">
         <is>
-          <t>.267</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" s="168" t="inlineStr">
         <is>
-          <t>.522</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O3" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -3350,57 +3350,57 @@
       </c>
       <c r="E4" s="168" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="168" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="168" t="inlineStr">
         <is>
-          <t>.300</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="168" t="inlineStr">
         <is>
-          <t>.417</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" s="168" t="inlineStr">
         <is>
-          <t>.575</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="168" t="inlineStr">
         <is>
-          <t>.992</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O4" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -3427,57 +3427,57 @@
       </c>
       <c r="E5" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="168" t="inlineStr">
         <is>
-          <t>.143</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L5" s="168" t="inlineStr">
         <is>
-          <t>.143</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" s="168" t="inlineStr">
         <is>
-          <t>.286</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" s="168" t="inlineStr">
         <is>
-          <t>.429</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O5" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -3504,57 +3504,57 @@
       </c>
       <c r="E6" s="168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="168" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="168" t="inlineStr">
         <is>
-          <t>.439</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="168" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="168" t="inlineStr">
         <is>
-          <t>.511</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" s="168" t="inlineStr">
         <is>
-          <t>1.098</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" s="168" t="inlineStr">
         <is>
-          <t>1.609</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="O7" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="O8" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -3735,57 +3735,57 @@
       </c>
       <c r="E9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="168" t="inlineStr">
         <is>
-          <t>.400</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="168" t="inlineStr">
         <is>
-          <t>.571</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M9" s="168" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N9" s="168" t="inlineStr">
         <is>
-          <t>1.771</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O9" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -3812,57 +3812,57 @@
       </c>
       <c r="E10" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="168" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="168" t="inlineStr">
         <is>
-          <t>.385</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="168" t="inlineStr">
         <is>
-          <t>.529</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="168" t="inlineStr">
         <is>
-          <t>.385</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="168" t="inlineStr">
         <is>
-          <t>.914</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O10" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="O11" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -3966,57 +3966,57 @@
       </c>
       <c r="E12" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="168" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="168" t="inlineStr">
         <is>
-          <t>.125</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M12" s="168" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="168" t="inlineStr">
         <is>
-          <t>.125</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O12" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4043,57 +4043,57 @@
       </c>
       <c r="E13" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" s="168" t="inlineStr">
         <is>
-          <t>.200</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K13" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L13" s="168" t="inlineStr">
         <is>
-          <t>.200</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M13" s="168" t="inlineStr">
         <is>
-          <t>.200</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" s="168" t="inlineStr">
         <is>
-          <t>.400</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O13" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4120,57 +4120,57 @@
       </c>
       <c r="E14" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" s="168" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" s="168" t="inlineStr">
         <is>
-          <t>.421</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J14" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L14" s="168" t="inlineStr">
         <is>
-          <t>.450</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M14" s="168" t="inlineStr">
         <is>
-          <t>.526</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N14" s="168" t="inlineStr">
         <is>
-          <t>.976</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O14" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="O15" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="O16" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4351,57 +4351,57 @@
       </c>
       <c r="E17" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="168" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N17" s="168" t="inlineStr">
         <is>
-          <t>.666</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O17" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="O18" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="O19" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4666,57 +4666,57 @@
       </c>
       <c r="E23" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="168" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="168" t="inlineStr">
         <is>
-          <t>0.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M23" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N23" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4743,57 +4743,57 @@
       </c>
       <c r="E24" s="168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I24" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J24" s="168" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K24" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L24" s="168" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M24" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N24" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O24" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4820,57 +4820,57 @@
       </c>
       <c r="E25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="168" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="168" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="168" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="168" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N25" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O25" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -4897,57 +4897,57 @@
       </c>
       <c r="E26" s="168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="168" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="168" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="168" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N26" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O26" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
       </c>
       <c r="O27" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5051,57 +5051,57 @@
       </c>
       <c r="E28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="168" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="168" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="168" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M28" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N28" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O28" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5128,57 +5128,57 @@
       </c>
       <c r="E29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J29" s="168" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K29" s="168" t="inlineStr">
         <is>
-          <t>10.57</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L29" s="168" t="inlineStr">
         <is>
-          <t>2.48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M29" s="168" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N29" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O29" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
       </c>
       <c r="O30" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5282,57 +5282,57 @@
       </c>
       <c r="E31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="168" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="168" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="168" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="168" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N31" s="168" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O31" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5359,57 +5359,57 @@
       </c>
       <c r="E32" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F32" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G32" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I32" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J32" s="168" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K32" s="168" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L32" s="168" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M32" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N32" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O32" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="O33" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="O34" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="O35" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O36" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       </c>
       <c r="O37" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="O38" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O39" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="O40" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -6052,57 +6052,57 @@
       </c>
       <c r="E41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F41" s="168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J41" s="168" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K41" s="168" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L41" s="168" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M41" s="168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N41" s="168" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O41" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="O42" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="O43" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>
@@ -6333,7 +6333,7 @@
       </c>
       <c r="O44" s="168" t="inlineStr">
         <is>
-          <t>04/08/2026 12:01</t>
+          <t>04/07/2026 15:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update roster: Drohan to MLB/Brewers, Maison Martinez season-ending injury
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6" yWindow="6" windowWidth="23028" windowHeight="13668" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$K$35</definedName>
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -94,15 +94,6 @@
       <color theme="10"/>
       <sz val="11"/>
       <u val="single"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="23">
@@ -265,7 +256,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -567,10 +558,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1255,12 +1242,12 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Nashville Sounds</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F9" s="11" t="n">
@@ -1280,7 +1267,7 @@
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>On 40-man roster; 2.27 ERA at Triple-A in 2025; called up to Boston Nov 2025, traded to MIL Feb 2026</t>
+          <t>MLB debut 2026 with Milwaukee Brewers; traded from BOS Feb 2026; previously 2.27 ERA at Triple-A in 2025</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2667,7 @@
       <c r="J38" s="43" t="n"/>
       <c r="K38" s="45" t="inlineStr">
         <is>
-          <t>2025 16th-round pick</t>
+          <t>2025 16th-round pick; injured, out for 2026 season</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -3037,105 +3024,96 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:O44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" style="89" min="1" max="1"/>
     <col width="8" customWidth="1" style="89" min="2" max="2"/>
     <col width="28" customWidth="1" style="89" min="3" max="3"/>
     <col width="12" customWidth="1" style="89" min="4" max="4"/>
-    <col width="8" customWidth="1" style="89" min="5" max="5"/>
-    <col width="8" customWidth="1" style="89" min="6" max="6"/>
-    <col width="8" customWidth="1" style="89" min="7" max="7"/>
-    <col width="8" customWidth="1" style="89" min="8" max="8"/>
-    <col width="8" customWidth="1" style="89" min="9" max="9"/>
-    <col width="8" customWidth="1" style="89" min="10" max="10"/>
-    <col width="8" customWidth="1" style="89" min="11" max="11"/>
-    <col width="8" customWidth="1" style="89" min="12" max="12"/>
-    <col width="8" customWidth="1" style="89" min="13" max="13"/>
-    <col width="8" customWidth="1" style="89" min="14" max="14"/>
+    <col width="8" customWidth="1" style="89" min="5" max="14"/>
     <col width="18" customWidth="1" style="89" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="104" t="inlineStr">
+      <c r="A1" s="92" t="inlineStr">
         <is>
           <t>⚾  HITTERS — 2026 Stats</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="105" t="inlineStr">
+      <c r="A2" s="85" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B2" s="105" t="inlineStr">
+      <c r="B2" s="85" t="inlineStr">
         <is>
           <t>Pos</t>
         </is>
       </c>
-      <c r="C2" s="105" t="inlineStr">
+      <c r="C2" s="85" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="D2" s="105" t="inlineStr">
+      <c r="D2" s="85" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="E2" s="105" t="inlineStr">
+      <c r="E2" s="85" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="F2" s="105" t="inlineStr">
+      <c r="F2" s="85" t="inlineStr">
         <is>
           <t>AB</t>
         </is>
       </c>
-      <c r="G2" s="105" t="inlineStr">
+      <c r="G2" s="85" t="inlineStr">
         <is>
           <t>AVG</t>
         </is>
       </c>
-      <c r="H2" s="105" t="inlineStr">
+      <c r="H2" s="85" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="I2" s="105" t="inlineStr">
+      <c r="I2" s="85" t="inlineStr">
         <is>
           <t>RBI</t>
         </is>
       </c>
-      <c r="J2" s="105" t="inlineStr">
+      <c r="J2" s="85" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="K2" s="105" t="inlineStr">
+      <c r="K2" s="85" t="inlineStr">
         <is>
           <t>SB</t>
         </is>
       </c>
-      <c r="L2" s="105" t="inlineStr">
+      <c r="L2" s="85" t="inlineStr">
         <is>
           <t>OBP</t>
         </is>
       </c>
-      <c r="M2" s="105" t="inlineStr">
+      <c r="M2" s="85" t="inlineStr">
         <is>
           <t>SLG</t>
         </is>
       </c>
-      <c r="N2" s="105" t="inlineStr">
+      <c r="N2" s="85" t="inlineStr">
         <is>
           <t>OPS</t>
         </is>
       </c>
-      <c r="O2" s="105" t="inlineStr">
+      <c r="O2" s="85" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
@@ -3164,57 +3142,57 @@
       </c>
       <c r="E3" s="87" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="87" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" s="87" t="inlineStr">
         <is>
-          <t>.198</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" s="87" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K3" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L3" s="87" t="inlineStr">
         <is>
-          <t>.281</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" s="87" t="inlineStr">
         <is>
-          <t>.386</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" s="87" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O3" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
@@ -3241,57 +3219,57 @@
       </c>
       <c r="E4" s="87" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="87" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="87" t="inlineStr">
         <is>
-          <t>.239</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="87" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="87" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="87" t="inlineStr">
         <is>
-          <t>.324</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" s="87" t="inlineStr">
         <is>
-          <t>.398</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="87" t="inlineStr">
         <is>
-          <t>.722</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O4" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
@@ -3318,57 +3296,57 @@
       </c>
       <c r="E5" s="87" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="87" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="87" t="inlineStr">
         <is>
-          <t>.208</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L5" s="87" t="inlineStr">
         <is>
-          <t>.269</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" s="87" t="inlineStr">
         <is>
-          <t>.229</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" s="87" t="inlineStr">
         <is>
-          <t>.498</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O5" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
@@ -3395,74 +3373,74 @@
       </c>
       <c r="E6" s="87" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="87" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="87" t="inlineStr">
         <is>
-          <t>.292</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="87" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="87" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="87" t="inlineStr">
         <is>
-          <t>.385</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" s="87" t="inlineStr">
         <is>
-          <t>.697</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" s="87" t="inlineStr">
         <is>
-          <t>1.082</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="86" t="inlineStr">
         <is>
-          <t>Colton Vincent</t>
+          <t>DJ Stewart</t>
         </is>
       </c>
       <c r="B7" s="86" t="inlineStr">
         <is>
-          <t>C/OF</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="C7" s="87" t="inlineStr">
         <is>
-          <t>El Paso Chihuahuas</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D7" s="87" t="inlineStr">
@@ -3472,151 +3450,151 @@
       </c>
       <c r="E7" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F7" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" s="87" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H7" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I7" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J7" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K7" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L7" s="87" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M7" s="87" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N7" s="87" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O7" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="86" t="inlineStr">
         <is>
-          <t>Marco Dinges</t>
+          <t>Colton Vincent</t>
         </is>
       </c>
       <c r="B8" s="86" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C/OF</t>
         </is>
       </c>
       <c r="C8" s="87" t="inlineStr">
         <is>
-          <t>Wisconsin Timber Rattlers</t>
+          <t>El Paso Chihuahuas</t>
         </is>
       </c>
       <c r="D8" s="87" t="inlineStr">
         <is>
-          <t>High-A</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="E8" s="87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F8" s="87" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G8" s="87" t="inlineStr">
         <is>
-          <t>.281</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I8" s="87" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J8" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K8" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L8" s="87" t="inlineStr">
         <is>
-          <t>.477</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M8" s="87" t="inlineStr">
         <is>
-          <t>.531</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N8" s="87" t="inlineStr">
         <is>
-          <t>1.008</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O8" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="86" t="inlineStr">
         <is>
-          <t>Jaime Ferrer</t>
+          <t>Marco Dinges</t>
         </is>
       </c>
       <c r="B9" s="86" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C9" s="87" t="inlineStr">
         <is>
-          <t>Cedar Rapids Kernels</t>
+          <t>Wisconsin Timber Rattlers</t>
         </is>
       </c>
       <c r="D9" s="87" t="inlineStr">
@@ -3626,64 +3604,64 @@
       </c>
       <c r="E9" s="87" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="87" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="87" t="inlineStr">
         <is>
-          <t>.279</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="87" t="inlineStr">
         <is>
-          <t>.456</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M9" s="87" t="inlineStr">
         <is>
-          <t>.442</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N9" s="87" t="inlineStr">
         <is>
-          <t>.898</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O9" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="86" t="inlineStr">
         <is>
-          <t>Gage Harrelson</t>
+          <t>Jaime Ferrer</t>
         </is>
       </c>
       <c r="B10" s="86" t="inlineStr">
@@ -3693,7 +3671,7 @@
       </c>
       <c r="C10" s="87" t="inlineStr">
         <is>
-          <t>Tri-City Dust Devils</t>
+          <t>Cedar Rapids Kernels</t>
         </is>
       </c>
       <c r="D10" s="87" t="inlineStr">
@@ -3703,918 +3681,918 @@
       </c>
       <c r="E10" s="87" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="87" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="87" t="inlineStr">
         <is>
-          <t>.313</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="87" t="inlineStr">
         <is>
-          <t>.500</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="87" t="inlineStr">
         <is>
-          <t>.375</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="87" t="inlineStr">
         <is>
-          <t>.875</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O10" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="86" t="inlineStr">
         <is>
-          <t>Alex Lodise</t>
+          <t>Yoel Tejeda Jr.</t>
         </is>
       </c>
       <c r="B11" s="86" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="C11" s="87" t="inlineStr">
         <is>
-          <t>Augusta GreenJackets</t>
+          <t>Wilmington Blue Rocks</t>
         </is>
       </c>
       <c r="D11" s="87" t="inlineStr">
         <is>
-          <t>Low-A</t>
+          <t>High-A</t>
         </is>
       </c>
       <c r="E11" s="87" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F11" s="87" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G11" s="87" t="inlineStr">
         <is>
-          <t>.254</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H11" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J11" s="87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K11" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L11" s="87" t="inlineStr">
         <is>
-          <t>.351</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M11" s="87" t="inlineStr">
         <is>
-          <t>.358</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N11" s="87" t="inlineStr">
         <is>
-          <t>.709</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O11" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="86" t="inlineStr">
         <is>
-          <t>Jaxson West</t>
+          <t>Drew Faurot</t>
         </is>
       </c>
       <c r="B12" s="86" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>2B</t>
         </is>
       </c>
       <c r="C12" s="87" t="inlineStr">
         <is>
-          <t>Dunedin Blue Jays</t>
+          <t>Beloit Sky Carp</t>
         </is>
       </c>
       <c r="D12" s="87" t="inlineStr">
         <is>
+          <t>High-A</t>
+        </is>
+      </c>
+      <c r="E12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O12" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="86" t="inlineStr">
+        <is>
+          <t>Gage Harrelson</t>
+        </is>
+      </c>
+      <c r="B13" s="86" t="inlineStr">
+        <is>
+          <t>OF</t>
+        </is>
+      </c>
+      <c r="C13" s="87" t="inlineStr">
+        <is>
+          <t>Tri-City Dust Devils</t>
+        </is>
+      </c>
+      <c r="D13" s="87" t="inlineStr">
+        <is>
+          <t>High-A</t>
+        </is>
+      </c>
+      <c r="E13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N13" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O13" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="86" t="inlineStr">
+        <is>
+          <t>Alex Lodise</t>
+        </is>
+      </c>
+      <c r="B14" s="86" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="C14" s="87" t="inlineStr">
+        <is>
+          <t>Augusta GreenJackets</t>
+        </is>
+      </c>
+      <c r="D14" s="87" t="inlineStr">
+        <is>
           <t>Low-A</t>
         </is>
       </c>
-      <c r="E12" s="87" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="F12" s="87" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="G12" s="87" t="inlineStr">
-        <is>
-          <t>.469</t>
-        </is>
-      </c>
-      <c r="H12" s="87" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I12" s="87" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="J12" s="87" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="K12" s="87" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="L12" s="87" t="inlineStr">
-        <is>
-          <t>.485</t>
-        </is>
-      </c>
-      <c r="M12" s="87" t="inlineStr">
-        <is>
-          <t>.625</t>
-        </is>
-      </c>
-      <c r="N12" s="87" t="inlineStr">
-        <is>
-          <t>1.110</t>
-        </is>
-      </c>
-      <c r="O12" s="87" t="inlineStr">
-        <is>
-          <t>04/23/2026 00:19</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="104" t="inlineStr">
-        <is>
-          <t>🎯  PITCHERS — 2026 Stats</t>
+      <c r="E14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N14" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O14" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="105" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B15" s="105" t="inlineStr">
-        <is>
-          <t>Pos</t>
-        </is>
-      </c>
-      <c r="C15" s="105" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="D15" s="105" t="inlineStr">
-        <is>
-          <t>Level</t>
-        </is>
-      </c>
-      <c r="E15" s="105" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F15" s="105" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="G15" s="105" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="H15" s="105" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I15" s="105" t="inlineStr">
-        <is>
-          <t>SV</t>
-        </is>
-      </c>
-      <c r="J15" s="105" t="inlineStr">
-        <is>
-          <t>IP</t>
-        </is>
-      </c>
-      <c r="K15" s="105" t="inlineStr">
-        <is>
-          <t>ERA</t>
-        </is>
-      </c>
-      <c r="L15" s="105" t="inlineStr">
-        <is>
-          <t>WHIP</t>
-        </is>
-      </c>
-      <c r="M15" s="105" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="N15" s="105" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="O15" s="105" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
+      <c r="A15" s="86" t="inlineStr">
+        <is>
+          <t>Gavin Adams</t>
+        </is>
+      </c>
+      <c r="B15" s="86" t="inlineStr">
+        <is>
+          <t>1B/OF</t>
+        </is>
+      </c>
+      <c r="C15" s="87" t="inlineStr">
+        <is>
+          <t>Bradenton Marauders</t>
+        </is>
+      </c>
+      <c r="D15" s="87" t="inlineStr">
+        <is>
+          <t>Low-A</t>
+        </is>
+      </c>
+      <c r="E15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N15" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O15" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="86" t="inlineStr">
         <is>
-          <t>Luke Weaver</t>
+          <t>Max Williams</t>
         </is>
       </c>
       <c r="B16" s="86" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="C16" s="87" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Jupiter Hammerheads</t>
         </is>
       </c>
       <c r="D16" s="87" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>Low-A</t>
         </is>
       </c>
       <c r="E16" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F16" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G16" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H16" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I16" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J16" s="87" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K16" s="87" t="inlineStr">
         <is>
-          <t>6.23</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L16" s="87" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M16" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N16" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O16" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="86" t="inlineStr">
         <is>
-          <t>Tyler Holton</t>
+          <t>Jaxson West</t>
         </is>
       </c>
       <c r="B17" s="86" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C17" s="87" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Dunedin Blue Jays</t>
         </is>
       </c>
       <c r="D17" s="87" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>Low-A</t>
         </is>
       </c>
       <c r="E17" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="87" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="87" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="87" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N17" s="87" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O17" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="86" t="inlineStr">
         <is>
-          <t>Parker Messick</t>
+          <t>Robby Martin Jr.</t>
         </is>
       </c>
       <c r="B18" s="86" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="C18" s="87" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Kane County Cougars</t>
         </is>
       </c>
       <c r="D18" s="87" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="E18" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F18" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G18" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H18" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I18" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J18" s="87" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K18" s="87" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L18" s="87" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M18" s="87" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N18" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O18" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="86" t="inlineStr">
         <is>
-          <t>Cole Sands</t>
+          <t>Drew Mendoza</t>
         </is>
       </c>
       <c r="B19" s="86" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>1B/3B</t>
         </is>
       </c>
       <c r="C19" s="87" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>High Point Rockers</t>
         </is>
       </c>
       <c r="D19" s="87" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="E19" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F19" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I19" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J19" s="87" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K19" s="87" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L19" s="87" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M19" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N19" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O19" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="86" t="inlineStr">
-        <is>
-          <t>Jack Anderson</t>
-        </is>
-      </c>
-      <c r="B20" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C20" s="87" t="inlineStr">
-        <is>
-          <t>Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="D20" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E20" s="87" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F20" s="87" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G20" s="87" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H20" s="87" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I20" s="87" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J20" s="87" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
-      </c>
-      <c r="K20" s="87" t="inlineStr">
-        <is>
-          <t>3.38</t>
-        </is>
-      </c>
-      <c r="L20" s="87" t="inlineStr">
-        <is>
-          <t>1.25</t>
-        </is>
-      </c>
-      <c r="M20" s="87" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="N20" s="87" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="O20" s="87" t="inlineStr">
-        <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="86" t="inlineStr">
-        <is>
-          <t>Shane Drohan</t>
-        </is>
-      </c>
-      <c r="B21" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C21" s="87" t="inlineStr">
-        <is>
-          <t>Nashville Sounds</t>
-        </is>
-      </c>
-      <c r="D21" s="87" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="E21" s="87" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F21" s="87" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G21" s="87" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H21" s="87" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I21" s="87" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J21" s="87" t="inlineStr">
-        <is>
-          <t>13.2</t>
-        </is>
-      </c>
-      <c r="K21" s="87" t="inlineStr">
-        <is>
-          <t>3.29</t>
-        </is>
-      </c>
-      <c r="L21" s="87" t="inlineStr">
-        <is>
-          <t>1.54</t>
-        </is>
-      </c>
-      <c r="M21" s="87" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="N21" s="87" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="O21" s="87" t="inlineStr">
-        <is>
-          <t>04/23/2026 00:19</t>
+      <c r="A21" s="92" t="inlineStr">
+        <is>
+          <t>🎯  PITCHERS — 2026 Stats</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="86" t="inlineStr">
-        <is>
-          <t>CJ Van Eyk</t>
-        </is>
-      </c>
-      <c r="B22" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C22" s="87" t="inlineStr">
-        <is>
-          <t>Buffalo Bisons</t>
-        </is>
-      </c>
-      <c r="D22" s="87" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="E22" s="87" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F22" s="87" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G22" s="87" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H22" s="87" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I22" s="87" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J22" s="87" t="inlineStr">
-        <is>
-          <t>18.1</t>
-        </is>
-      </c>
-      <c r="K22" s="87" t="inlineStr">
-        <is>
-          <t>3.44</t>
-        </is>
-      </c>
-      <c r="L22" s="87" t="inlineStr">
-        <is>
-          <t>1.42</t>
-        </is>
-      </c>
-      <c r="M22" s="87" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="N22" s="87" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="O22" s="87" t="inlineStr">
-        <is>
-          <t>04/23/2026 00:19</t>
+      <c r="A22" s="85" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B22" s="85" t="inlineStr">
+        <is>
+          <t>Pos</t>
+        </is>
+      </c>
+      <c r="C22" s="85" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="D22" s="85" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="E22" s="85" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F22" s="85" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="G22" s="85" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H22" s="85" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I22" s="85" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="J22" s="85" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="K22" s="85" t="inlineStr">
+        <is>
+          <t>ERA</t>
+        </is>
+      </c>
+      <c r="L22" s="85" t="inlineStr">
+        <is>
+          <t>WHIP</t>
+        </is>
+      </c>
+      <c r="M22" s="85" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="N22" s="85" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="O22" s="85" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="86" t="inlineStr">
         <is>
-          <t>Brandon Leibrandt</t>
+          <t>Luke Weaver</t>
         </is>
       </c>
       <c r="B23" s="86" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C23" s="87" t="inlineStr">
         <is>
-          <t>Louisville Bats</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D23" s="87" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E23" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="87" t="inlineStr">
         <is>
-          <t>16.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="87" t="inlineStr">
         <is>
-          <t>5.51</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="87" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M23" s="87" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N23" s="87" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="86" t="inlineStr">
         <is>
-          <t>Drew Parrish</t>
+          <t>Tyler Holton</t>
         </is>
       </c>
       <c r="B24" s="86" t="inlineStr">
@@ -4624,12 +4602,12 @@
       </c>
       <c r="C24" s="87" t="inlineStr">
         <is>
-          <t>Louisville Bats</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D24" s="87" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E24" s="87" t="inlineStr">
@@ -4684,14 +4662,14 @@
       </c>
       <c r="O24" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="86" t="inlineStr">
         <is>
-          <t>Jamie Arnold</t>
+          <t>Parker Messick</t>
         </is>
       </c>
       <c r="B25" s="86" t="inlineStr">
@@ -4701,74 +4679,74 @@
       </c>
       <c r="C25" s="87" t="inlineStr">
         <is>
-          <t>Midland RockHounds</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="D25" s="87" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E25" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="87" t="inlineStr">
         <is>
-          <t>17.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="87" t="inlineStr">
         <is>
-          <t>2.55</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="87" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="87" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N25" s="87" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O25" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="86" t="inlineStr">
         <is>
-          <t>Jackson Baumeister</t>
+          <t>Cole Sands</t>
         </is>
       </c>
       <c r="B26" s="86" t="inlineStr">
@@ -4778,151 +4756,151 @@
       </c>
       <c r="C26" s="87" t="inlineStr">
         <is>
-          <t>Montgomery Biscuits</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D26" s="87" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E26" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="87" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="87" t="inlineStr">
         <is>
-          <t>5.79</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="87" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N26" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O26" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="86" t="inlineStr">
         <is>
-          <t>Wyatt Crowell</t>
+          <t>Jack Anderson</t>
         </is>
       </c>
       <c r="B27" s="86" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C27" s="87" t="inlineStr">
         <is>
-          <t>Tulsa Drillers</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="D27" s="87" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E27" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" s="87" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K27" s="87" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L27" s="87" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M27" s="87" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N27" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O27" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="86" t="inlineStr">
         <is>
-          <t>Carson Dorsey</t>
+          <t>Shane Drohan</t>
         </is>
       </c>
       <c r="B28" s="86" t="inlineStr">
@@ -4932,89 +4910,89 @@
       </c>
       <c r="C28" s="87" t="inlineStr">
         <is>
-          <t>Aberdeen IronBirds</t>
+          <t>Nashville Sounds</t>
         </is>
       </c>
       <c r="D28" s="87" t="inlineStr">
         <is>
-          <t>High-A</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="E28" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="87" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="87" t="inlineStr">
         <is>
-          <t>8.53</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="87" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M28" s="87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N28" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O28" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="86" t="inlineStr">
         <is>
-          <t>Conner Whittaker</t>
+          <t>CJ Van Eyk</t>
         </is>
       </c>
       <c r="B29" s="86" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C29" s="87" t="inlineStr">
         <is>
-          <t>Lake County Captains</t>
+          <t>Buffalo Bisons</t>
         </is>
       </c>
       <c r="D29" s="87" t="inlineStr">
         <is>
-          <t>High-A</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="E29" s="87" t="inlineStr">
@@ -5069,14 +5047,14 @@
       </c>
       <c r="O29" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="86" t="inlineStr">
         <is>
-          <t>Joey Volini</t>
+          <t>Brandon Leibrandt</t>
         </is>
       </c>
       <c r="B30" s="86" t="inlineStr">
@@ -5086,166 +5064,166 @@
       </c>
       <c r="C30" s="87" t="inlineStr">
         <is>
-          <t>Beloit Sky Carp</t>
+          <t>Louisville Bats</t>
         </is>
       </c>
       <c r="D30" s="87" t="inlineStr">
         <is>
-          <t>High-A</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="E30" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F30" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I30" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J30" s="87" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K30" s="87" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L30" s="87" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M30" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N30" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O30" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="86" t="inlineStr">
         <is>
-          <t>Gavin Adams</t>
+          <t>Drew Parrish</t>
         </is>
       </c>
       <c r="B31" s="86" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="C31" s="87" t="inlineStr">
         <is>
-          <t>Bradenton Marauders</t>
+          <t>Louisville Bats</t>
         </is>
       </c>
       <c r="D31" s="87" t="inlineStr">
         <is>
-          <t>Low-A</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="E31" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="87" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="87" t="inlineStr">
         <is>
-          <t>8.53</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="87" t="inlineStr">
         <is>
-          <t>2.53</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N31" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O31" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="86" t="inlineStr">
         <is>
-          <t>Yoel Tejeda Jr.</t>
+          <t>Jamie Arnold</t>
         </is>
       </c>
       <c r="B32" s="86" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="C32" s="87" t="inlineStr">
         <is>
-          <t>Wilmington Blue Rocks</t>
+          <t>Midland RockHounds</t>
         </is>
       </c>
       <c r="D32" s="87" t="inlineStr">
         <is>
-          <t>Low-A</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="E32" s="87" t="inlineStr">
@@ -5300,91 +5278,91 @@
       </c>
       <c r="O32" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="86" t="inlineStr">
         <is>
-          <t>Bryce Hubbart</t>
+          <t>Jackson Baumeister</t>
         </is>
       </c>
       <c r="B33" s="86" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C33" s="87" t="inlineStr">
         <is>
-          <t>Daytona Tortugas</t>
+          <t>Montgomery Biscuits</t>
         </is>
       </c>
       <c r="D33" s="87" t="inlineStr">
         <is>
-          <t>Low-A</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="E33" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F33" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G33" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J33" s="87" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K33" s="87" t="inlineStr">
         <is>
-          <t>6.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L33" s="87" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M33" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N33" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O33" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="86" t="inlineStr">
         <is>
-          <t>Carson Montgomery</t>
+          <t>J.C. Flowers</t>
         </is>
       </c>
       <c r="B34" s="86" t="inlineStr">
@@ -5394,12 +5372,12 @@
       </c>
       <c r="C34" s="87" t="inlineStr">
         <is>
-          <t>Fort Wayne TinCaps</t>
+          <t>Altoona Curve</t>
         </is>
       </c>
       <c r="D34" s="87" t="inlineStr">
         <is>
-          <t>Low-A</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="E34" s="87" t="inlineStr">
@@ -5454,168 +5432,784 @@
       </c>
       <c r="O34" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="86" t="inlineStr">
         <is>
-          <t>Cam Leiter</t>
+          <t>Carson Dorsey</t>
         </is>
       </c>
       <c r="B35" s="86" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="C35" s="87" t="inlineStr">
         <is>
-          <t>Ontario Tower Buzzers</t>
+          <t>Aberdeen IronBirds</t>
         </is>
       </c>
       <c r="D35" s="87" t="inlineStr">
         <is>
-          <t>Low-A</t>
+          <t>High-A</t>
         </is>
       </c>
       <c r="E35" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F35" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G35" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H35" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I35" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J35" s="87" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K35" s="87" t="inlineStr">
         <is>
-          <t>3.86</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L35" s="87" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M35" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N35" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O35" s="87" t="inlineStr">
         <is>
-          <t>04/23/2026 00:19</t>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="86" t="inlineStr">
         <is>
+          <t>Wyatt Crowell</t>
+        </is>
+      </c>
+      <c r="B36" s="86" t="inlineStr">
+        <is>
+          <t>LHP</t>
+        </is>
+      </c>
+      <c r="C36" s="87" t="inlineStr">
+        <is>
+          <t>Great Lakes Loons</t>
+        </is>
+      </c>
+      <c r="D36" s="87" t="inlineStr">
+        <is>
+          <t>High-A</t>
+        </is>
+      </c>
+      <c r="E36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N36" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O36" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="86" t="inlineStr">
+        <is>
+          <t>Conner Whittaker</t>
+        </is>
+      </c>
+      <c r="B37" s="86" t="inlineStr">
+        <is>
+          <t>LHP</t>
+        </is>
+      </c>
+      <c r="C37" s="87" t="inlineStr">
+        <is>
+          <t>Lake County Captains</t>
+        </is>
+      </c>
+      <c r="D37" s="87" t="inlineStr">
+        <is>
+          <t>High-A</t>
+        </is>
+      </c>
+      <c r="E37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N37" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O37" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="86" t="inlineStr">
+        <is>
+          <t>Joey Volini</t>
+        </is>
+      </c>
+      <c r="B38" s="86" t="inlineStr">
+        <is>
+          <t>LHP</t>
+        </is>
+      </c>
+      <c r="C38" s="87" t="inlineStr">
+        <is>
+          <t>Beloit Sky Carp</t>
+        </is>
+      </c>
+      <c r="D38" s="87" t="inlineStr">
+        <is>
+          <t>High-A</t>
+        </is>
+      </c>
+      <c r="E38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N38" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O38" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="86" t="inlineStr">
+        <is>
+          <t>Bryce Hubbart</t>
+        </is>
+      </c>
+      <c r="B39" s="86" t="inlineStr">
+        <is>
+          <t>LHP</t>
+        </is>
+      </c>
+      <c r="C39" s="87" t="inlineStr">
+        <is>
+          <t>Daytona Tortugas</t>
+        </is>
+      </c>
+      <c r="D39" s="87" t="inlineStr">
+        <is>
+          <t>Low-A</t>
+        </is>
+      </c>
+      <c r="E39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N39" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O39" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="86" t="inlineStr">
+        <is>
+          <t>Carson Montgomery</t>
+        </is>
+      </c>
+      <c r="B40" s="86" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
+      <c r="C40" s="87" t="inlineStr">
+        <is>
+          <t>Fort Wayne TinCaps</t>
+        </is>
+      </c>
+      <c r="D40" s="87" t="inlineStr">
+        <is>
+          <t>Low-A</t>
+        </is>
+      </c>
+      <c r="E40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N40" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O40" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="86" t="inlineStr">
+        <is>
+          <t>Cam Leiter</t>
+        </is>
+      </c>
+      <c r="B41" s="86" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
+      <c r="C41" s="87" t="inlineStr">
+        <is>
+          <t>Ontario Tower Buzzers</t>
+        </is>
+      </c>
+      <c r="D41" s="87" t="inlineStr">
+        <is>
+          <t>Low-A</t>
+        </is>
+      </c>
+      <c r="E41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N41" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O41" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="86" t="inlineStr">
+        <is>
+          <t>Peyton Prescott</t>
+        </is>
+      </c>
+      <c r="B42" s="86" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
+      <c r="C42" s="87" t="inlineStr">
+        <is>
+          <t>ACL/AZL</t>
+        </is>
+      </c>
+      <c r="D42" s="87" t="inlineStr">
+        <is>
+          <t>Rookie</t>
+        </is>
+      </c>
+      <c r="E42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N42" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O42" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="86" t="inlineStr">
+        <is>
           <t>Evan Chrest</t>
         </is>
       </c>
-      <c r="B36" s="86" t="inlineStr">
+      <c r="B43" s="86" t="inlineStr">
         <is>
           <t>RHP</t>
         </is>
       </c>
-      <c r="C36" s="87" t="inlineStr">
+      <c r="C43" s="87" t="inlineStr">
         <is>
           <t>ACL/AZL</t>
         </is>
       </c>
-      <c r="D36" s="87" t="inlineStr">
+      <c r="D43" s="87" t="inlineStr">
         <is>
           <t>Rookie</t>
         </is>
       </c>
-      <c r="E36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O36" s="87" t="inlineStr">
-        <is>
-          <t>04/23/2026 00:19</t>
+      <c r="E43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N43" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O43" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="86" t="inlineStr">
+        <is>
+          <t>Maison Martinez</t>
+        </is>
+      </c>
+      <c r="B44" s="86" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
+      <c r="C44" s="87" t="inlineStr">
+        <is>
+          <t>ACL/AZL</t>
+        </is>
+      </c>
+      <c r="D44" s="87" t="inlineStr">
+        <is>
+          <t>Rookie</t>
+        </is>
+      </c>
+      <c r="E44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N44" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O44" s="87" t="inlineStr">
+        <is>
+          <t>04/14/2026 18:09</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A14:O14"/>
+    <mergeCell ref="A21:O21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Joe Charles (RHP, Brooklyn Cyclones High-A) to roster
- Added Joe Charles to noles_in_the_pros.xlsx Roster sheet
  (New York Mets org, High-A Brooklyn Cyclones, 2019 Rd 25 Pick #748)
- Updated noles_stats_updater.py to also write index.html on each run
  so beyondhowser.com stays in sync automatically going forward
- Added Joe Charles player ID (683087) to player_id_cache.json
- Regenerated index.html and noles_dashboard.html with Joe Charles included

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6" yWindow="6" windowWidth="23028" windowHeight="13668" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$K$35</definedName>
@@ -832,7 +832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" style="89" min="1" max="1"/>
@@ -1904,921 +1904,967 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="89">
-      <c r="A23" s="26" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Joe Charles</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>RHP</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>High-A</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Brooklyn Cyclones</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G23" t="n">
+        <v>25</v>
+      </c>
+      <c r="H23" t="n">
+        <v>748</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://www.milb.com/player/joe-charles-683087</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2019 25th-round pick; signed as FA by Mets Aug 2025 after FSU career; promoted to High-A Brooklyn April 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="89">
+      <c r="A24" s="26" t="inlineStr">
         <is>
           <t>Wyatt Crowell</t>
         </is>
       </c>
-      <c r="B23" s="27" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>LHP</t>
         </is>
       </c>
-      <c r="C23" s="27" t="inlineStr">
+      <c r="C24" s="27" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="D23" s="27" t="inlineStr">
+      <c r="D24" s="27" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="E23" s="28" t="inlineStr">
+      <c r="E24" s="28" t="inlineStr">
         <is>
           <t>Tulsa Drillers</t>
         </is>
       </c>
-      <c r="F23" s="27" t="n">
+      <c r="F24" s="27" t="n">
         <v>2023</v>
       </c>
-      <c r="G23" s="27" t="n">
+      <c r="G24" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="H23" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I23" s="27" t="n"/>
-      <c r="J23" s="102" t="inlineStr">
+      <c r="H24" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="27" t="n"/>
+      <c r="J24" s="102" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/wyatt-crowell-694573</t>
         </is>
       </c>
-      <c r="K23" s="29" t="inlineStr">
+      <c r="K24" s="29" t="inlineStr">
         <is>
           <t>Returned from Tommy John in 2025; mid-80s slider with ~50% whiff rate</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1" s="89">
-      <c r="A24" s="34" t="inlineStr">
+    <row r="25" ht="18" customHeight="1" s="89">
+      <c r="A25" s="34" t="inlineStr">
         <is>
           <t>Gavin Adams</t>
         </is>
       </c>
-      <c r="B24" s="35" t="inlineStr">
+      <c r="B25" s="35" t="inlineStr">
         <is>
           <t>RHP</t>
         </is>
       </c>
-      <c r="C24" s="35" t="inlineStr">
+      <c r="C25" s="35" t="inlineStr">
         <is>
           <t>Pittsburgh Pirates</t>
         </is>
       </c>
-      <c r="D24" s="35" t="inlineStr">
+      <c r="D25" s="35" t="inlineStr">
         <is>
           <t>Low-A</t>
         </is>
       </c>
-      <c r="E24" s="36" t="inlineStr">
+      <c r="E25" s="36" t="inlineStr">
         <is>
           <t>Bradenton Marauders</t>
         </is>
       </c>
-      <c r="F24" s="35" t="n">
+      <c r="F25" s="35" t="n">
         <v>2024</v>
       </c>
-      <c r="G24" s="35" t="n">
+      <c r="G25" s="35" t="n">
         <v>8</v>
       </c>
-      <c r="H24" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="35" t="n"/>
-      <c r="J24" s="103" t="inlineStr">
+      <c r="H25" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="35" t="n"/>
+      <c r="J25" s="103" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/gavin-adams-701400</t>
         </is>
       </c>
-      <c r="K24" s="37" t="inlineStr">
+      <c r="K25" s="37" t="inlineStr">
         <is>
           <t>2024 8th-round pick</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1" s="89">
-      <c r="A25" s="38" t="inlineStr">
+    <row r="26" ht="18" customHeight="1" s="89">
+      <c r="A26" s="38" t="inlineStr">
         <is>
           <t>Yoel Tejeda Jr.</t>
         </is>
       </c>
-      <c r="B25" s="39" t="inlineStr">
+      <c r="B26" s="39" t="inlineStr">
         <is>
           <t>RHP</t>
         </is>
       </c>
-      <c r="C25" s="39" t="inlineStr">
+      <c r="C26" s="39" t="inlineStr">
         <is>
           <t>Washington Nationals</t>
         </is>
       </c>
-      <c r="D25" s="39" t="inlineStr">
+      <c r="D26" s="39" t="inlineStr">
         <is>
           <t>Low-A</t>
         </is>
       </c>
-      <c r="E25" s="40" t="inlineStr">
+      <c r="E26" s="40" t="inlineStr">
         <is>
           <t>Wilmington Blue Rocks</t>
         </is>
       </c>
-      <c r="F25" s="39" t="n">
+      <c r="F26" s="39" t="n">
         <v>2024</v>
       </c>
-      <c r="G25" s="39" t="n">
+      <c r="G26" s="39" t="n">
         <v>14</v>
       </c>
-      <c r="H25" s="39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" s="39" t="n"/>
-      <c r="J25" s="39" t="inlineStr">
+      <c r="H26" s="39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="39" t="n"/>
+      <c r="J26" s="39" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/yoel-tejeda-jr-701347</t>
         </is>
       </c>
-      <c r="K25" s="41" t="inlineStr">
+      <c r="K26" s="41" t="inlineStr">
         <is>
           <t>2024 14th-round pick</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1" s="89">
-      <c r="A26" s="34" t="inlineStr">
+    <row r="27" ht="18" customHeight="1" s="89">
+      <c r="A27" s="34" t="inlineStr">
         <is>
           <t>Conner Whittaker</t>
         </is>
       </c>
-      <c r="B26" s="35" t="inlineStr">
+      <c r="B27" s="35" t="inlineStr">
         <is>
           <t>LHP</t>
         </is>
       </c>
-      <c r="C26" s="35" t="inlineStr">
+      <c r="C27" s="35" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="D26" s="35" t="inlineStr">
+      <c r="D27" s="35" t="inlineStr">
         <is>
           <t>High-A</t>
         </is>
       </c>
-      <c r="E26" s="36" t="inlineStr">
+      <c r="E27" s="36" t="inlineStr">
         <is>
           <t>Lake County Captains</t>
         </is>
       </c>
-      <c r="F26" s="35" t="n">
+      <c r="F27" s="35" t="n">
         <v>2024</v>
       </c>
-      <c r="G26" s="35" t="n">
+      <c r="G27" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="H26" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="35" t="n"/>
-      <c r="J26" s="35" t="inlineStr">
+      <c r="H27" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="35" t="n"/>
+      <c r="J27" s="35" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/conner-whittaker-701422</t>
         </is>
       </c>
-      <c r="K26" s="37" t="inlineStr">
+      <c r="K27" s="37" t="inlineStr">
         <is>
           <t>2024 15th-round pick</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1" s="89">
-      <c r="A27" s="38" t="inlineStr">
+    <row r="28" ht="18" customHeight="1" s="89">
+      <c r="A28" s="38" t="inlineStr">
         <is>
           <t>Bryce Hubbart</t>
         </is>
       </c>
-      <c r="B27" s="39" t="inlineStr">
+      <c r="B28" s="39" t="inlineStr">
         <is>
           <t>LHP</t>
         </is>
       </c>
-      <c r="C27" s="39" t="inlineStr">
+      <c r="C28" s="39" t="inlineStr">
         <is>
           <t>Cincinnati Reds</t>
         </is>
       </c>
-      <c r="D27" s="39" t="inlineStr">
+      <c r="D28" s="39" t="inlineStr">
         <is>
           <t>Low-A</t>
         </is>
       </c>
-      <c r="E27" s="40" t="inlineStr">
+      <c r="E28" s="40" t="inlineStr">
         <is>
           <t>Daytona Tortugas</t>
         </is>
       </c>
-      <c r="F27" s="39" t="n">
+      <c r="F28" s="39" t="n">
         <v>2022</v>
       </c>
-      <c r="G27" s="39" t="n">
+      <c r="G28" s="39" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="39" t="n">
+      <c r="H28" s="39" t="n">
         <v>94</v>
       </c>
-      <c r="I27" s="39" t="n"/>
-      <c r="J27" s="39" t="inlineStr">
+      <c r="I28" s="39" t="n"/>
+      <c r="J28" s="39" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/bryce-hubbart-687114</t>
         </is>
       </c>
-      <c r="K27" s="41" t="inlineStr">
+      <c r="K28" s="41" t="inlineStr">
         <is>
           <t>Deceptive high-spin southpaw; working through Reds system</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1" s="89">
-      <c r="A28" s="34" t="inlineStr">
+    <row r="29" ht="18" customHeight="1" s="89">
+      <c r="A29" s="34" t="inlineStr">
         <is>
           <t>Carson Montgomery</t>
         </is>
       </c>
-      <c r="B28" s="35" t="inlineStr">
+      <c r="B29" s="35" t="inlineStr">
         <is>
           <t>RHP</t>
         </is>
       </c>
-      <c r="C28" s="35" t="inlineStr">
+      <c r="C29" s="35" t="inlineStr">
         <is>
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="D28" s="35" t="inlineStr">
+      <c r="D29" s="35" t="inlineStr">
         <is>
           <t>Low-A</t>
         </is>
       </c>
-      <c r="E28" s="36" t="inlineStr">
+      <c r="E29" s="36" t="inlineStr">
         <is>
           <t>Fort Wayne TinCaps</t>
         </is>
       </c>
-      <c r="F28" s="35" t="n">
+      <c r="F29" s="35" t="n">
         <v>2023</v>
       </c>
-      <c r="G28" s="35" t="n">
+      <c r="G29" s="35" t="n">
         <v>11</v>
       </c>
-      <c r="H28" s="35" t="n">
+      <c r="H29" s="35" t="n">
         <v>341</v>
       </c>
-      <c r="I28" s="35" t="n"/>
-      <c r="J28" s="35" t="inlineStr">
+      <c r="I29" s="35" t="n"/>
+      <c r="J29" s="35" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/carson-montgomery-691000</t>
         </is>
       </c>
-      <c r="K28" s="37" t="inlineStr">
+      <c r="K29" s="37" t="inlineStr">
         <is>
           <t>97-98 mph FB, nasty slider; 2025 Arizona Fall League participant</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1" s="89">
-      <c r="A29" s="81" t="inlineStr">
+    <row r="30" ht="18" customHeight="1" s="89">
+      <c r="A30" s="81" t="inlineStr">
         <is>
           <t>Colton Vincent</t>
         </is>
       </c>
-      <c r="B29" s="82" t="inlineStr">
+      <c r="B30" s="82" t="inlineStr">
         <is>
           <t>C/OF</t>
         </is>
       </c>
-      <c r="C29" s="82" t="inlineStr">
+      <c r="C30" s="82" t="inlineStr">
         <is>
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="D29" s="82" t="inlineStr">
+      <c r="D30" s="82" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="E29" s="83" t="inlineStr">
+      <c r="E30" s="83" t="inlineStr">
         <is>
           <t>El Paso Chihuahuas</t>
         </is>
       </c>
-      <c r="F29" s="82" t="n">
+      <c r="F30" s="82" t="n">
         <v>2023</v>
       </c>
-      <c r="G29" s="82" t="inlineStr">
+      <c r="G30" s="82" t="inlineStr">
         <is>
           <t>UDFA</t>
         </is>
       </c>
-      <c r="H29" s="82" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I29" s="82" t="n"/>
-      <c r="J29" s="82" t="inlineStr">
+      <c r="H30" s="82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I30" s="82" t="n"/>
+      <c r="J30" s="82" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/colton-vincent-694294</t>
         </is>
       </c>
-      <c r="K29" s="84" t="inlineStr">
+      <c r="K30" s="84" t="inlineStr">
         <is>
           <t>Undrafted free agent 2023; versatile C/OF/1B; .827 OPS in 40+ games at Peoria Low-A in 2025; in Lake Elsinore catching rotation for 2026</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1" s="89">
-      <c r="A30" s="42" t="inlineStr">
+    <row r="31" ht="18" customHeight="1" s="89">
+      <c r="A31" s="42" t="inlineStr">
         <is>
           <t>Max Williams</t>
         </is>
       </c>
-      <c r="B30" s="43" t="inlineStr">
+      <c r="B31" s="43" t="inlineStr">
         <is>
           <t>OF</t>
         </is>
       </c>
-      <c r="C30" s="43" t="inlineStr">
+      <c r="C31" s="43" t="inlineStr">
         <is>
           <t>Miami Marlins</t>
         </is>
       </c>
-      <c r="D30" s="43" t="inlineStr">
+      <c r="D31" s="43" t="inlineStr">
         <is>
           <t>60-Day IL</t>
         </is>
       </c>
-      <c r="E30" s="44" t="inlineStr">
+      <c r="E31" s="44" t="inlineStr">
         <is>
           <t>Jupiter Hammerheads</t>
         </is>
       </c>
-      <c r="F30" s="43" t="n">
+      <c r="F31" s="43" t="n">
         <v>2025</v>
       </c>
-      <c r="G30" s="43" t="n">
+      <c r="G31" s="43" t="n">
         <v>3</v>
       </c>
-      <c r="H30" s="43" t="n">
+      <c r="H31" s="43" t="n">
         <v>78</v>
       </c>
-      <c r="I30" s="43" t="n"/>
-      <c r="J30" s="43" t="inlineStr">
+      <c r="I31" s="43" t="n"/>
+      <c r="J31" s="43" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/max-williams-703637</t>
         </is>
       </c>
-      <c r="K30" s="45" t="inlineStr">
+      <c r="K31" s="45" t="inlineStr">
         <is>
           <t>.321/19HR/.990 OPS at FSU; hit .316 with 6HR in pro debut at Low-A Jupiter</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>Low-A</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1" s="89">
-      <c r="A31" s="46" t="inlineStr">
+    <row r="32" ht="18" customHeight="1" s="89">
+      <c r="A32" s="46" t="inlineStr">
         <is>
           <t>Drew Faurot</t>
         </is>
       </c>
-      <c r="B31" s="47" t="inlineStr">
+      <c r="B32" s="47" t="inlineStr">
         <is>
           <t>2B</t>
         </is>
       </c>
-      <c r="C31" s="47" t="inlineStr">
+      <c r="C32" s="47" t="inlineStr">
         <is>
           <t>Miami Marlins</t>
         </is>
       </c>
-      <c r="D31" s="47" t="inlineStr">
+      <c r="D32" s="47" t="inlineStr">
         <is>
           <t>7-Day IL</t>
         </is>
       </c>
-      <c r="E31" s="48" t="inlineStr">
+      <c r="E32" s="48" t="inlineStr">
         <is>
           <t>Beloit Sky Carp</t>
         </is>
       </c>
-      <c r="F31" s="47" t="n">
+      <c r="F32" s="47" t="n">
         <v>2025</v>
       </c>
-      <c r="G31" s="47" t="n">
+      <c r="G32" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="H31" s="47" t="n">
+      <c r="H32" s="47" t="n">
         <v>108</v>
       </c>
-      <c r="I31" s="47" t="n"/>
-      <c r="J31" s="47" t="inlineStr">
+      <c r="I32" s="47" t="n"/>
+      <c r="J32" s="47" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/drew-faurot-702656</t>
         </is>
       </c>
-      <c r="K31" s="49" t="inlineStr">
+      <c r="K32" s="49" t="inlineStr">
         <is>
           <t>Tallahassee native; .307/16HR/.952 OPS at FSU; 3-for-3 pro debut; 25% below slot signing</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>High-A</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1" s="89">
-      <c r="A32" s="42" t="inlineStr">
+    <row r="33" ht="18" customHeight="1" s="89">
+      <c r="A33" s="42" t="inlineStr">
         <is>
           <t>Joey Volini</t>
         </is>
       </c>
-      <c r="B32" s="43" t="inlineStr">
+      <c r="B33" s="43" t="inlineStr">
         <is>
           <t>LHP</t>
         </is>
       </c>
-      <c r="C32" s="43" t="inlineStr">
+      <c r="C33" s="43" t="inlineStr">
         <is>
           <t>Miami Marlins</t>
         </is>
       </c>
-      <c r="D32" s="43" t="inlineStr">
+      <c r="D33" s="43" t="inlineStr">
         <is>
           <t>High-A</t>
         </is>
       </c>
-      <c r="E32" s="44" t="inlineStr">
+      <c r="E33" s="44" t="inlineStr">
         <is>
           <t>Beloit Sky Carp</t>
         </is>
       </c>
-      <c r="F32" s="43" t="n">
+      <c r="F33" s="43" t="n">
         <v>2025</v>
       </c>
-      <c r="G32" s="43" t="n">
+      <c r="G33" s="43" t="n">
         <v>6</v>
       </c>
-      <c r="H32" s="43" t="n">
+      <c r="H33" s="43" t="n">
         <v>168</v>
       </c>
-      <c r="I32" s="43" t="n"/>
-      <c r="J32" s="43" t="inlineStr">
+      <c r="I33" s="43" t="n"/>
+      <c r="J33" s="43" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/joey-volini-804123</t>
         </is>
       </c>
-      <c r="K32" s="45" t="inlineStr">
+      <c r="K33" s="45" t="inlineStr">
         <is>
           <t>Dick Howser National Pitcher of Month (March 2025); 8-5, 3.50 ERA, 105K at FSU; TJ survivor</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1" s="89">
-      <c r="A33" s="46" t="inlineStr">
+    <row r="34" ht="18" customHeight="1" s="89">
+      <c r="A34" s="46" t="inlineStr">
         <is>
           <t>Cam Leiter</t>
         </is>
       </c>
-      <c r="B33" s="47" t="inlineStr">
+      <c r="B34" s="47" t="inlineStr">
         <is>
           <t>RHP</t>
         </is>
       </c>
-      <c r="C33" s="47" t="inlineStr">
+      <c r="C34" s="47" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="D33" s="47" t="inlineStr">
+      <c r="D34" s="47" t="inlineStr">
         <is>
           <t>Low-A</t>
         </is>
       </c>
-      <c r="E33" s="48" t="inlineStr">
+      <c r="E34" s="48" t="inlineStr">
         <is>
           <t>Ontario Tower Buzzers</t>
         </is>
       </c>
-      <c r="F33" s="47" t="n">
+      <c r="F34" s="47" t="n">
         <v>2025</v>
       </c>
-      <c r="G33" s="47" t="n">
+      <c r="G34" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="H33" s="47" t="n">
+      <c r="H34" s="47" t="n">
         <v>65</v>
       </c>
-      <c r="I33" s="47" t="n"/>
-      <c r="J33" s="47" t="inlineStr">
+      <c r="I34" s="47" t="n"/>
+      <c r="J34" s="47" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/cam-leiter-804942</t>
         </is>
       </c>
-      <c r="K33" s="49" t="inlineStr">
+      <c r="K34" s="49" t="inlineStr">
         <is>
           <t>Dealing with injury post-draft; 2026 assignment TBD on recovery</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1" s="89">
-      <c r="A34" s="42" t="inlineStr">
+    <row r="35" ht="18" customHeight="1" s="89">
+      <c r="A35" s="42" t="inlineStr">
         <is>
           <t>Peyton Prescott</t>
         </is>
       </c>
-      <c r="B34" s="43" t="inlineStr">
+      <c r="B35" s="43" t="inlineStr">
         <is>
           <t>RHP</t>
         </is>
       </c>
-      <c r="C34" s="43" t="inlineStr">
+      <c r="C35" s="43" t="inlineStr">
         <is>
           <t>New York Mets</t>
         </is>
       </c>
-      <c r="D34" s="43" t="inlineStr">
+      <c r="D35" s="43" t="inlineStr">
         <is>
           <t>60-Day IL</t>
         </is>
       </c>
-      <c r="E34" s="44" t="inlineStr">
+      <c r="E35" s="44" t="inlineStr">
         <is>
           <t>ACL/AZL</t>
         </is>
       </c>
-      <c r="F34" s="43" t="n">
+      <c r="F35" s="43" t="n">
         <v>2025</v>
       </c>
-      <c r="G34" s="43" t="n">
+      <c r="G35" s="43" t="n">
         <v>5</v>
       </c>
-      <c r="H34" s="43" t="n">
+      <c r="H35" s="43" t="n">
         <v>163</v>
       </c>
-      <c r="I34" s="43" t="n"/>
-      <c r="J34" s="43" t="inlineStr">
+      <c r="I35" s="43" t="n"/>
+      <c r="J35" s="43" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/peyton-prescott-807290</t>
         </is>
       </c>
-      <c r="K34" s="45" t="inlineStr">
+      <c r="K35" s="45" t="inlineStr">
         <is>
           <t>Dealing with injury post-draft</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>Rookie</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1" s="89">
-      <c r="A35" s="46" t="inlineStr">
+    <row r="36" ht="14.4" customHeight="1" s="89">
+      <c r="A36" s="46" t="inlineStr">
         <is>
           <t>Evan Chrest</t>
         </is>
       </c>
-      <c r="B35" s="47" t="inlineStr">
+      <c r="B36" s="47" t="inlineStr">
         <is>
           <t>RHP</t>
         </is>
       </c>
-      <c r="C35" s="47" t="inlineStr">
+      <c r="C36" s="47" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="D35" s="47" t="inlineStr">
+      <c r="D36" s="47" t="inlineStr">
         <is>
           <t>Rookie</t>
         </is>
       </c>
-      <c r="E35" s="48" t="inlineStr">
+      <c r="E36" s="48" t="inlineStr">
         <is>
           <t>ACL/AZL</t>
         </is>
       </c>
-      <c r="F35" s="47" t="n">
+      <c r="F36" s="47" t="n">
         <v>2025</v>
       </c>
-      <c r="G35" s="47" t="n">
+      <c r="G36" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="H35" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="47" t="n"/>
-      <c r="J35" s="47" t="inlineStr">
+      <c r="H36" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="47" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/evan-chrest-805971</t>
         </is>
       </c>
-      <c r="K35" s="49" t="inlineStr">
+      <c r="K36" s="49" t="inlineStr">
         <is>
           <t>2025 15th-round pick</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="14.4" customHeight="1" s="89">
-      <c r="A36" s="42" t="inlineStr">
+    <row r="37" ht="14.4" customHeight="1" s="89">
+      <c r="A37" s="42" t="inlineStr">
         <is>
           <t>Gage Harrelson</t>
         </is>
       </c>
-      <c r="B36" s="43" t="inlineStr">
+      <c r="B37" s="43" t="inlineStr">
         <is>
           <t>OF</t>
         </is>
       </c>
-      <c r="C36" s="43" t="inlineStr">
+      <c r="C37" s="43" t="inlineStr">
         <is>
           <t>Los Angeles Angels</t>
         </is>
       </c>
-      <c r="D36" s="43" t="inlineStr">
+      <c r="D37" s="43" t="inlineStr">
         <is>
           <t>High-A</t>
         </is>
       </c>
-      <c r="E36" s="44" t="inlineStr">
+      <c r="E37" s="44" t="inlineStr">
         <is>
           <t>Tri-City Dust Devils</t>
         </is>
       </c>
-      <c r="F36" s="43" t="n">
+      <c r="F37" s="43" t="n">
         <v>2025</v>
       </c>
-      <c r="G36" s="43" t="n">
+      <c r="G37" s="43" t="n">
         <v>16</v>
       </c>
-      <c r="H36" s="43" t="n">
+      <c r="H37" s="43" t="n">
         <v>469</v>
       </c>
-      <c r="I36" s="43" t="n"/>
-      <c r="J36" s="43" t="inlineStr">
+      <c r="I37" s="43" t="n"/>
+      <c r="J37" s="43" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/gage-harrelson-702629</t>
         </is>
       </c>
-      <c r="K36" s="45" t="inlineStr">
+      <c r="K37" s="45" t="inlineStr">
         <is>
           <t>.339/.444/.462, 15 SB at FSU; plus speed, projects as CF; signed $150K</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="14.4" customHeight="1" s="89">
-      <c r="A37" s="46" t="inlineStr">
+    <row r="38" ht="14.4" customHeight="1" s="89">
+      <c r="A38" s="46" t="inlineStr">
         <is>
           <t>Jaxson West</t>
         </is>
       </c>
-      <c r="B37" s="47" t="inlineStr">
+      <c r="B38" s="47" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C37" s="47" t="inlineStr">
+      <c r="C38" s="47" t="inlineStr">
         <is>
           <t>Toronto Blue Jays</t>
         </is>
       </c>
-      <c r="D37" s="47" t="inlineStr">
+      <c r="D38" s="47" t="inlineStr">
         <is>
           <t>Low-A</t>
         </is>
       </c>
-      <c r="E37" s="48" t="inlineStr">
+      <c r="E38" s="48" t="inlineStr">
         <is>
           <t>Dunedin Blue Jays</t>
         </is>
       </c>
-      <c r="F37" s="47" t="n">
+      <c r="F38" s="47" t="n">
         <v>2025</v>
       </c>
-      <c r="G37" s="47" t="n">
+      <c r="G38" s="47" t="n">
         <v>16</v>
       </c>
-      <c r="H37" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I37" s="47" t="n"/>
-      <c r="J37" s="47" t="inlineStr">
+      <c r="H38" s="47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="47" t="n"/>
+      <c r="J38" s="47" t="inlineStr">
         <is>
           <t>https://www.mlb.com/player/jaxson-west-702486</t>
         </is>
       </c>
-      <c r="K37" s="49" t="inlineStr">
+      <c r="K38" s="49" t="inlineStr">
         <is>
           <t>2025 16th-round pick</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="14.4" customHeight="1" s="89">
-      <c r="A38" s="42" t="inlineStr">
+    <row r="39" ht="24.6" customHeight="1" s="89">
+      <c r="A39" s="42" t="inlineStr">
         <is>
           <t>Maison Martinez</t>
         </is>
       </c>
-      <c r="B38" s="43" t="inlineStr">
+      <c r="B39" s="43" t="inlineStr">
         <is>
           <t>RHP</t>
         </is>
       </c>
-      <c r="C38" s="43" t="inlineStr">
+      <c r="C39" s="43" t="inlineStr">
         <is>
           <t>Cincinnati Reds</t>
         </is>
       </c>
-      <c r="D38" s="43" t="inlineStr">
+      <c r="D39" s="43" t="inlineStr">
         <is>
           <t>60-Day IL</t>
         </is>
       </c>
-      <c r="E38" s="44" t="inlineStr">
+      <c r="E39" s="44" t="inlineStr">
         <is>
           <t>ACL/AZL</t>
         </is>
       </c>
-      <c r="F38" s="43" t="n">
+      <c r="F39" s="43" t="n">
         <v>2025</v>
       </c>
-      <c r="G38" s="43" t="n">
+      <c r="G39" s="43" t="n">
         <v>16</v>
       </c>
-      <c r="H38" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I38" s="43" t="n"/>
-      <c r="J38" s="43" t="n"/>
-      <c r="K38" s="45" t="inlineStr">
+      <c r="H39" s="43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" s="43" t="n"/>
+      <c r="J39" s="43" t="n"/>
+      <c r="K39" s="45" t="inlineStr">
         <is>
           <t>2025 16th-round pick; injured, out for 2026 season</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>Rookie</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="24.6" customHeight="1" s="89">
-      <c r="A39" s="50" t="inlineStr">
+    <row r="40" ht="24.6" customHeight="1" s="89">
+      <c r="A40" s="50" t="inlineStr">
         <is>
           <t>Robby Martin Jr.</t>
         </is>
       </c>
-      <c r="B39" s="51" t="inlineStr">
+      <c r="B40" s="51" t="inlineStr">
         <is>
           <t>OF</t>
         </is>
       </c>
-      <c r="C39" s="51" t="inlineStr">
+      <c r="C40" s="51" t="inlineStr">
         <is>
           <t>Kane County Cougars</t>
         </is>
       </c>
-      <c r="D39" s="51" t="inlineStr">
+      <c r="D40" s="51" t="inlineStr">
         <is>
           <t>Independent</t>
         </is>
       </c>
-      <c r="E39" s="52" t="inlineStr">
+      <c r="E40" s="52" t="inlineStr">
         <is>
           <t>Kane County Cougars</t>
         </is>
       </c>
-      <c r="F39" s="51" t="n">
+      <c r="F40" s="51" t="n">
         <v>2021</v>
       </c>
-      <c r="G39" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H39" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I39" s="51" t="n"/>
-      <c r="J39" s="51" t="n"/>
-      <c r="K39" s="53" t="inlineStr">
+      <c r="G40" s="51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I40" s="51" t="n"/>
+      <c r="J40" s="51" t="n"/>
+      <c r="K40" s="53" t="inlineStr">
         <is>
           <t>Released by Rockies March 2025; .198/.265/.320, 6HR in 59G with Kane County (American Association)</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="24.6" customHeight="1" s="89">
-      <c r="A40" s="54" t="inlineStr">
+    <row r="41" ht="36.9" customHeight="1" s="89">
+      <c r="A41" s="54" t="inlineStr">
         <is>
           <t>Matheu Nelson</t>
         </is>
       </c>
-      <c r="B40" s="55" t="inlineStr">
+      <c r="B41" s="55" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C40" s="55" t="inlineStr">
+      <c r="C41" s="55" t="inlineStr">
         <is>
           <t>Lake Country DockHounds</t>
         </is>
       </c>
-      <c r="D40" s="55" t="inlineStr">
+      <c r="D41" s="55" t="inlineStr">
         <is>
           <t>Independent</t>
         </is>
       </c>
-      <c r="E40" s="56" t="inlineStr">
+      <c r="E41" s="56" t="inlineStr">
         <is>
           <t>Lake Country DockHounds</t>
         </is>
       </c>
-      <c r="F40" s="55" t="n">
+      <c r="F41" s="55" t="n">
         <v>2021</v>
       </c>
-      <c r="G40" s="55" t="inlineStr">
+      <c r="G41" s="55" t="inlineStr">
         <is>
           <t>CB-A</t>
         </is>
       </c>
-      <c r="H40" s="55" t="n">
+      <c r="H41" s="55" t="n">
         <v>35</v>
       </c>
-      <c r="I40" s="55" t="n"/>
-      <c r="J40" s="55" t="n"/>
-      <c r="K40" s="57" t="inlineStr">
+      <c r="I41" s="55" t="n"/>
+      <c r="J41" s="55" t="n"/>
+      <c r="K41" s="57" t="inlineStr">
         <is>
           <t>Former #35 overall pick (Reds); ACC POY at FSU; released by CIN July 2025 after .088 BA at Double-A</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="36.9" customHeight="1" s="89">
-      <c r="A41" s="50" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="50" t="inlineStr">
         <is>
           <t>Drew Mendoza</t>
         </is>
       </c>
-      <c r="B41" s="51" t="inlineStr">
+      <c r="B42" s="51" t="inlineStr">
         <is>
           <t>1B/3B</t>
         </is>
       </c>
-      <c r="C41" s="51" t="inlineStr">
+      <c r="C42" s="51" t="inlineStr">
         <is>
           <t>High Point Rockers</t>
         </is>
       </c>
-      <c r="D41" s="51" t="inlineStr">
+      <c r="D42" s="51" t="inlineStr">
         <is>
           <t>Independent</t>
         </is>
       </c>
-      <c r="E41" s="52" t="inlineStr">
+      <c r="E42" s="52" t="inlineStr">
         <is>
           <t>High Point Rockers</t>
         </is>
       </c>
-      <c r="F41" s="51" t="n">
+      <c r="F42" s="51" t="n">
         <v>2019</v>
       </c>
-      <c r="G41" s="51" t="n">
+      <c r="G42" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="H41" s="51" t="n">
+      <c r="H42" s="51" t="n">
         <v>94</v>
       </c>
-      <c r="I41" s="51" t="n"/>
-      <c r="J41" s="51" t="n"/>
-      <c r="K41" s="53" t="inlineStr">
+      <c r="I42" s="51" t="n"/>
+      <c r="J42" s="51" t="n"/>
+      <c r="K42" s="53" t="inlineStr">
         <is>
           <t>Former Nationals 3rd-round pick; 2023 ALPB batting champ (.346, York Revolution); named to 2025 ALPB All-Star team with High Point Rockers; 2026 status TBD</t>
         </is>
@@ -3164,57 +3210,57 @@
       </c>
       <c r="E3" s="87" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="87" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" s="87" t="inlineStr">
         <is>
-          <t>.198</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I3" s="87" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K3" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L3" s="87" t="inlineStr">
         <is>
-          <t>.281</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M3" s="87" t="inlineStr">
         <is>
-          <t>.386</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N3" s="87" t="inlineStr">
         <is>
-          <t>.667</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O3" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -3241,57 +3287,57 @@
       </c>
       <c r="E4" s="87" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="87" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" s="87" t="inlineStr">
         <is>
-          <t>.239</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I4" s="87" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="87" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="87" t="inlineStr">
         <is>
-          <t>.324</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M4" s="87" t="inlineStr">
         <is>
-          <t>.398</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="87" t="inlineStr">
         <is>
-          <t>.722</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O4" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -3318,57 +3364,57 @@
       </c>
       <c r="E5" s="87" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="87" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="87" t="inlineStr">
         <is>
-          <t>.208</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I5" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K5" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L5" s="87" t="inlineStr">
         <is>
-          <t>.269</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" s="87" t="inlineStr">
         <is>
-          <t>.229</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" s="87" t="inlineStr">
         <is>
-          <t>.498</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O5" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -3395,57 +3441,57 @@
       </c>
       <c r="E6" s="87" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="87" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" s="87" t="inlineStr">
         <is>
-          <t>.295</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="87" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="87" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K6" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="87" t="inlineStr">
         <is>
-          <t>.393</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M6" s="87" t="inlineStr">
         <is>
-          <t>.705</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N6" s="87" t="inlineStr">
         <is>
-          <t>1.098</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O6" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -3472,57 +3518,57 @@
       </c>
       <c r="E7" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F7" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" s="87" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H7" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I7" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J7" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K7" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L7" s="87" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M7" s="87" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N7" s="87" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O7" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -3549,57 +3595,57 @@
       </c>
       <c r="E8" s="87" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F8" s="87" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G8" s="87" t="inlineStr">
         <is>
-          <t>.268</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I8" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J8" s="87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K8" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L8" s="87" t="inlineStr">
         <is>
-          <t>.455</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M8" s="87" t="inlineStr">
         <is>
-          <t>.537</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N8" s="87" t="inlineStr">
         <is>
-          <t>.992</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O8" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -3626,57 +3672,57 @@
       </c>
       <c r="E9" s="87" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="87" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" s="87" t="inlineStr">
         <is>
-          <t>.283</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I9" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K9" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L9" s="87" t="inlineStr">
         <is>
-          <t>.459</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M9" s="87" t="inlineStr">
         <is>
-          <t>.435</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N9" s="87" t="inlineStr">
         <is>
-          <t>.894</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O9" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -3703,57 +3749,57 @@
       </c>
       <c r="E10" s="87" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="87" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" s="87" t="inlineStr">
         <is>
-          <t>.278</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I10" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="87" t="inlineStr">
         <is>
-          <t>.480</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="87" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="87" t="inlineStr">
         <is>
-          <t>.813</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O10" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -3780,57 +3826,57 @@
       </c>
       <c r="E11" s="87" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F11" s="87" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G11" s="87" t="inlineStr">
         <is>
-          <t>.276</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H11" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J11" s="87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K11" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L11" s="87" t="inlineStr">
         <is>
-          <t>.360</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M11" s="87" t="inlineStr">
         <is>
-          <t>.395</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N11" s="87" t="inlineStr">
         <is>
-          <t>.755</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O11" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -3857,57 +3903,57 @@
       </c>
       <c r="E12" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="87" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" s="87" t="inlineStr">
         <is>
-          <t>.469</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I12" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L12" s="87" t="inlineStr">
         <is>
-          <t>.485</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M12" s="87" t="inlineStr">
         <is>
-          <t>.625</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="87" t="inlineStr">
         <is>
-          <t>1.110</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O12" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4018,57 +4064,57 @@
       </c>
       <c r="E16" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F16" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G16" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H16" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I16" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J16" s="87" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K16" s="87" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L16" s="87" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M16" s="87" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N16" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O16" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4095,57 +4141,57 @@
       </c>
       <c r="E17" s="87" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F17" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H17" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J17" s="87" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="87" t="inlineStr">
         <is>
-          <t>3.27</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="87" t="inlineStr">
         <is>
-          <t>1.64</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N17" s="87" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O17" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4172,57 +4218,57 @@
       </c>
       <c r="E18" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F18" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G18" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H18" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I18" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J18" s="87" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K18" s="87" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L18" s="87" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M18" s="87" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N18" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O18" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4249,57 +4295,57 @@
       </c>
       <c r="E19" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F19" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I19" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J19" s="87" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K19" s="87" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L19" s="87" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M19" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N19" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O19" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4326,57 +4372,57 @@
       </c>
       <c r="E20" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F20" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G20" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I20" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J20" s="87" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K20" s="87" t="inlineStr">
         <is>
-          <t>10.13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L20" s="87" t="inlineStr">
         <is>
-          <t>2.63</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M20" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N20" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O20" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4403,57 +4449,57 @@
       </c>
       <c r="E21" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F21" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G21" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H21" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I21" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J21" s="87" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K21" s="87" t="inlineStr">
         <is>
-          <t>3.38</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L21" s="87" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M21" s="87" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N21" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O21" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4480,57 +4526,57 @@
       </c>
       <c r="E22" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F22" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G22" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H22" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I22" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J22" s="87" t="inlineStr">
         <is>
-          <t>18.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K22" s="87" t="inlineStr">
         <is>
-          <t>3.44</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L22" s="87" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M22" s="87" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N22" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O22" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4557,57 +4603,57 @@
       </c>
       <c r="E23" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I23" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J23" s="87" t="inlineStr">
         <is>
-          <t>16.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K23" s="87" t="inlineStr">
         <is>
-          <t>5.51</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L23" s="87" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M23" s="87" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N23" s="87" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4684,7 +4730,7 @@
       </c>
       <c r="O24" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4711,57 +4757,57 @@
       </c>
       <c r="E25" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J25" s="87" t="inlineStr">
         <is>
-          <t>17.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K25" s="87" t="inlineStr">
         <is>
-          <t>2.55</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L25" s="87" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M25" s="87" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N25" s="87" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O25" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4788,57 +4834,57 @@
       </c>
       <c r="E26" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F26" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J26" s="87" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K26" s="87" t="inlineStr">
         <is>
-          <t>5.79</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L26" s="87" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N26" s="87" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O26" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4865,57 +4911,57 @@
       </c>
       <c r="E27" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J27" s="87" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K27" s="87" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L27" s="87" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M27" s="87" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N27" s="87" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O27" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -4942,57 +4988,57 @@
       </c>
       <c r="E28" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G28" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J28" s="87" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="87" t="inlineStr">
         <is>
-          <t>8.53</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="87" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M28" s="87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N28" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O28" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -5069,7 +5115,7 @@
       </c>
       <c r="O29" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -5096,57 +5142,57 @@
       </c>
       <c r="E30" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F30" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I30" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J30" s="87" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K30" s="87" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L30" s="87" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M30" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N30" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O30" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -5173,57 +5219,57 @@
       </c>
       <c r="E31" s="87" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G31" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J31" s="87" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K31" s="87" t="inlineStr">
         <is>
-          <t>7.36</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L31" s="87" t="inlineStr">
         <is>
-          <t>2.18</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M31" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N31" s="87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O31" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5346,7 @@
       </c>
       <c r="O32" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -5327,57 +5373,57 @@
       </c>
       <c r="E33" s="87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F33" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G33" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J33" s="87" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K33" s="87" t="inlineStr">
         <is>
-          <t>6.75</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L33" s="87" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M33" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N33" s="87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O33" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5500,7 @@
       </c>
       <c r="O34" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -5481,57 +5527,57 @@
       </c>
       <c r="E35" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F35" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G35" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H35" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I35" s="87" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J35" s="87" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K35" s="87" t="inlineStr">
         <is>
-          <t>3.86</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L35" s="87" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M35" s="87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N35" s="87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O35" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5654,7 @@
       </c>
       <c r="O36" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 12:06</t>
+          <t>04/24/2026 20:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Maison Martinez to Full Season IL
- Changed level from 60-Day IL to Full Season IL in roster Excel and site HTML
- Updated notes: out for full 2026 season
- Added Full Season IL as a recognized level in noles_stats_updater.py
  (skips API lookup, shown in special section with IL badge)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -2703,12 +2703,12 @@
       </c>
       <c r="D39" s="43" t="inlineStr">
         <is>
-          <t>60-Day IL</t>
+          <t>Full Season IL</t>
         </is>
       </c>
       <c r="E39" s="44" t="inlineStr">
         <is>
-          <t>ACL/AZL</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F39" s="43" t="n">
@@ -2726,7 +2726,7 @@
       <c r="J39" s="43" t="n"/>
       <c r="K39" s="45" t="inlineStr">
         <is>
-          <t>2025 16th-round pick; injured, out for 2026 season</t>
+          <t>2025 16th-round pick; out for full 2026 season (injury)</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3083,7 +3083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="89" min="1" max="1"/>
@@ -3187,2481 +3187,171 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="86" t="inlineStr">
-        <is>
-          <t>Cal Raleigh</t>
-        </is>
-      </c>
-      <c r="B3" s="86" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C3" s="87" t="inlineStr">
-        <is>
-          <t>Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="D3" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O3" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
     <row r="4">
-      <c r="A4" s="86" t="inlineStr">
-        <is>
-          <t>Cam Smith</t>
-        </is>
-      </c>
-      <c r="B4" s="86" t="inlineStr">
-        <is>
-          <t>OF/3B</t>
-        </is>
-      </c>
-      <c r="C4" s="87" t="inlineStr">
-        <is>
-          <t>Houston Astros</t>
-        </is>
-      </c>
-      <c r="D4" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N4" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O4" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
+      <c r="A4" s="104" t="inlineStr">
+        <is>
+          <t>🎯  PITCHERS — 2026 Stats</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="86" t="inlineStr">
-        <is>
-          <t>Taylor Walls</t>
-        </is>
-      </c>
-      <c r="B5" s="86" t="inlineStr">
-        <is>
-          <t>SS</t>
-        </is>
-      </c>
-      <c r="C5" s="87" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="D5" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N5" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O5" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
+      <c r="A5" s="105" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B5" s="105" t="inlineStr">
+        <is>
+          <t>Pos</t>
+        </is>
+      </c>
+      <c r="C5" s="105" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="D5" s="105" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="E5" s="105" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F5" s="105" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="G5" s="105" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H5" s="105" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I5" s="105" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="J5" s="105" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="K5" s="105" t="inlineStr">
+        <is>
+          <t>ERA</t>
+        </is>
+      </c>
+      <c r="L5" s="105" t="inlineStr">
+        <is>
+          <t>WHIP</t>
+        </is>
+      </c>
+      <c r="M5" s="105" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="N5" s="105" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="O5" s="105" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="86" t="inlineStr">
         <is>
-          <t>James Tibbs III</t>
+          <t>Joe Charles</t>
         </is>
       </c>
       <c r="B6" s="86" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C6" s="87" t="inlineStr">
         <is>
-          <t>Oklahoma City Comets</t>
+          <t>Brooklyn Cyclones</t>
         </is>
       </c>
       <c r="D6" s="87" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>High-A</t>
         </is>
       </c>
       <c r="E6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="K6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.46</t>
         </is>
       </c>
       <c r="L6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.31</t>
         </is>
       </c>
       <c r="M6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N6" s="87" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7</t>
         </is>
       </c>
       <c r="O6" s="87" t="inlineStr">
         <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="86" t="inlineStr">
-        <is>
-          <t>Colton Vincent</t>
-        </is>
-      </c>
-      <c r="B7" s="86" t="inlineStr">
-        <is>
-          <t>C/OF</t>
-        </is>
-      </c>
-      <c r="C7" s="87" t="inlineStr">
-        <is>
-          <t>El Paso Chihuahuas</t>
-        </is>
-      </c>
-      <c r="D7" s="87" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="E7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N7" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O7" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="86" t="inlineStr">
-        <is>
-          <t>Marco Dinges</t>
-        </is>
-      </c>
-      <c r="B8" s="86" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C8" s="87" t="inlineStr">
-        <is>
-          <t>Wisconsin Timber Rattlers</t>
-        </is>
-      </c>
-      <c r="D8" s="87" t="inlineStr">
-        <is>
-          <t>High-A</t>
-        </is>
-      </c>
-      <c r="E8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N8" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O8" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="86" t="inlineStr">
-        <is>
-          <t>Jaime Ferrer</t>
-        </is>
-      </c>
-      <c r="B9" s="86" t="inlineStr">
-        <is>
-          <t>OF</t>
-        </is>
-      </c>
-      <c r="C9" s="87" t="inlineStr">
-        <is>
-          <t>Cedar Rapids Kernels</t>
-        </is>
-      </c>
-      <c r="D9" s="87" t="inlineStr">
-        <is>
-          <t>High-A</t>
-        </is>
-      </c>
-      <c r="E9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N9" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O9" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="86" t="inlineStr">
-        <is>
-          <t>Gage Harrelson</t>
-        </is>
-      </c>
-      <c r="B10" s="86" t="inlineStr">
-        <is>
-          <t>OF</t>
-        </is>
-      </c>
-      <c r="C10" s="87" t="inlineStr">
-        <is>
-          <t>Tri-City Dust Devils</t>
-        </is>
-      </c>
-      <c r="D10" s="87" t="inlineStr">
-        <is>
-          <t>High-A</t>
-        </is>
-      </c>
-      <c r="E10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N10" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O10" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="86" t="inlineStr">
-        <is>
-          <t>Alex Lodise</t>
-        </is>
-      </c>
-      <c r="B11" s="86" t="inlineStr">
-        <is>
-          <t>SS</t>
-        </is>
-      </c>
-      <c r="C11" s="87" t="inlineStr">
-        <is>
-          <t>Augusta GreenJackets</t>
-        </is>
-      </c>
-      <c r="D11" s="87" t="inlineStr">
-        <is>
-          <t>Low-A</t>
-        </is>
-      </c>
-      <c r="E11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N11" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O11" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="86" t="inlineStr">
-        <is>
-          <t>Jaxson West</t>
-        </is>
-      </c>
-      <c r="B12" s="86" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C12" s="87" t="inlineStr">
-        <is>
-          <t>Dunedin Blue Jays</t>
-        </is>
-      </c>
-      <c r="D12" s="87" t="inlineStr">
-        <is>
-          <t>Low-A</t>
-        </is>
-      </c>
-      <c r="E12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N12" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O12" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="104" t="inlineStr">
-        <is>
-          <t>🎯  PITCHERS — 2026 Stats</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="105" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B15" s="105" t="inlineStr">
-        <is>
-          <t>Pos</t>
-        </is>
-      </c>
-      <c r="C15" s="105" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="D15" s="105" t="inlineStr">
-        <is>
-          <t>Level</t>
-        </is>
-      </c>
-      <c r="E15" s="105" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F15" s="105" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="G15" s="105" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="H15" s="105" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I15" s="105" t="inlineStr">
-        <is>
-          <t>SV</t>
-        </is>
-      </c>
-      <c r="J15" s="105" t="inlineStr">
-        <is>
-          <t>IP</t>
-        </is>
-      </c>
-      <c r="K15" s="105" t="inlineStr">
-        <is>
-          <t>ERA</t>
-        </is>
-      </c>
-      <c r="L15" s="105" t="inlineStr">
-        <is>
-          <t>WHIP</t>
-        </is>
-      </c>
-      <c r="M15" s="105" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="N15" s="105" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="O15" s="105" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="86" t="inlineStr">
-        <is>
-          <t>Luke Weaver</t>
-        </is>
-      </c>
-      <c r="B16" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C16" s="87" t="inlineStr">
-        <is>
-          <t>New York Mets</t>
-        </is>
-      </c>
-      <c r="D16" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N16" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O16" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="86" t="inlineStr">
-        <is>
-          <t>Tyler Holton</t>
-        </is>
-      </c>
-      <c r="B17" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C17" s="87" t="inlineStr">
-        <is>
-          <t>Detroit Tigers</t>
-        </is>
-      </c>
-      <c r="D17" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N17" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O17" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="86" t="inlineStr">
-        <is>
-          <t>Parker Messick</t>
-        </is>
-      </c>
-      <c r="B18" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C18" s="87" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="D18" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N18" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O18" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="86" t="inlineStr">
-        <is>
-          <t>Cole Sands</t>
-        </is>
-      </c>
-      <c r="B19" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C19" s="87" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="D19" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N19" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O19" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="86" t="inlineStr">
-        <is>
-          <t>Shane Drohan</t>
-        </is>
-      </c>
-      <c r="B20" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C20" s="87" t="inlineStr">
-        <is>
-          <t>Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="D20" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N20" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O20" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="86" t="inlineStr">
-        <is>
-          <t>Jack Anderson</t>
-        </is>
-      </c>
-      <c r="B21" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C21" s="87" t="inlineStr">
-        <is>
-          <t>Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="D21" s="87" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N21" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O21" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="86" t="inlineStr">
-        <is>
-          <t>CJ Van Eyk</t>
-        </is>
-      </c>
-      <c r="B22" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C22" s="87" t="inlineStr">
-        <is>
-          <t>Buffalo Bisons</t>
-        </is>
-      </c>
-      <c r="D22" s="87" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="E22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N22" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O22" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="86" t="inlineStr">
-        <is>
-          <t>Brandon Leibrandt</t>
-        </is>
-      </c>
-      <c r="B23" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C23" s="87" t="inlineStr">
-        <is>
-          <t>Louisville Bats</t>
-        </is>
-      </c>
-      <c r="D23" s="87" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="E23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N23" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O23" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="86" t="inlineStr">
-        <is>
-          <t>Drew Parrish</t>
-        </is>
-      </c>
-      <c r="B24" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C24" s="87" t="inlineStr">
-        <is>
-          <t>Louisville Bats</t>
-        </is>
-      </c>
-      <c r="D24" s="87" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="E24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N24" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O24" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="86" t="inlineStr">
-        <is>
-          <t>Jamie Arnold</t>
-        </is>
-      </c>
-      <c r="B25" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C25" s="87" t="inlineStr">
-        <is>
-          <t>Midland RockHounds</t>
-        </is>
-      </c>
-      <c r="D25" s="87" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="E25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N25" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O25" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="86" t="inlineStr">
-        <is>
-          <t>Jackson Baumeister</t>
-        </is>
-      </c>
-      <c r="B26" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C26" s="87" t="inlineStr">
-        <is>
-          <t>Montgomery Biscuits</t>
-        </is>
-      </c>
-      <c r="D26" s="87" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="E26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N26" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O26" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="86" t="inlineStr">
-        <is>
-          <t>Wyatt Crowell</t>
-        </is>
-      </c>
-      <c r="B27" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C27" s="87" t="inlineStr">
-        <is>
-          <t>Tulsa Drillers</t>
-        </is>
-      </c>
-      <c r="D27" s="87" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="E27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N27" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O27" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="86" t="inlineStr">
-        <is>
-          <t>Carson Dorsey</t>
-        </is>
-      </c>
-      <c r="B28" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C28" s="87" t="inlineStr">
-        <is>
-          <t>Aberdeen IronBirds</t>
-        </is>
-      </c>
-      <c r="D28" s="87" t="inlineStr">
-        <is>
-          <t>High-A</t>
-        </is>
-      </c>
-      <c r="E28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N28" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O28" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="86" t="inlineStr">
-        <is>
-          <t>Conner Whittaker</t>
-        </is>
-      </c>
-      <c r="B29" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C29" s="87" t="inlineStr">
-        <is>
-          <t>Lake County Captains</t>
-        </is>
-      </c>
-      <c r="D29" s="87" t="inlineStr">
-        <is>
-          <t>High-A</t>
-        </is>
-      </c>
-      <c r="E29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N29" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O29" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="86" t="inlineStr">
-        <is>
-          <t>Joey Volini</t>
-        </is>
-      </c>
-      <c r="B30" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C30" s="87" t="inlineStr">
-        <is>
-          <t>Beloit Sky Carp</t>
-        </is>
-      </c>
-      <c r="D30" s="87" t="inlineStr">
-        <is>
-          <t>High-A</t>
-        </is>
-      </c>
-      <c r="E30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N30" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O30" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="86" t="inlineStr">
-        <is>
-          <t>Gavin Adams</t>
-        </is>
-      </c>
-      <c r="B31" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C31" s="87" t="inlineStr">
-        <is>
-          <t>Bradenton Marauders</t>
-        </is>
-      </c>
-      <c r="D31" s="87" t="inlineStr">
-        <is>
-          <t>Low-A</t>
-        </is>
-      </c>
-      <c r="E31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N31" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O31" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="86" t="inlineStr">
-        <is>
-          <t>Yoel Tejeda Jr.</t>
-        </is>
-      </c>
-      <c r="B32" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C32" s="87" t="inlineStr">
-        <is>
-          <t>Wilmington Blue Rocks</t>
-        </is>
-      </c>
-      <c r="D32" s="87" t="inlineStr">
-        <is>
-          <t>Low-A</t>
-        </is>
-      </c>
-      <c r="E32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N32" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O32" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="86" t="inlineStr">
-        <is>
-          <t>Bryce Hubbart</t>
-        </is>
-      </c>
-      <c r="B33" s="86" t="inlineStr">
-        <is>
-          <t>LHP</t>
-        </is>
-      </c>
-      <c r="C33" s="87" t="inlineStr">
-        <is>
-          <t>Daytona Tortugas</t>
-        </is>
-      </c>
-      <c r="D33" s="87" t="inlineStr">
-        <is>
-          <t>Low-A</t>
-        </is>
-      </c>
-      <c r="E33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N33" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O33" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="86" t="inlineStr">
-        <is>
-          <t>Carson Montgomery</t>
-        </is>
-      </c>
-      <c r="B34" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C34" s="87" t="inlineStr">
-        <is>
-          <t>Fort Wayne TinCaps</t>
-        </is>
-      </c>
-      <c r="D34" s="87" t="inlineStr">
-        <is>
-          <t>Low-A</t>
-        </is>
-      </c>
-      <c r="E34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N34" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O34" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="86" t="inlineStr">
-        <is>
-          <t>Cam Leiter</t>
-        </is>
-      </c>
-      <c r="B35" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C35" s="87" t="inlineStr">
-        <is>
-          <t>Ontario Tower Buzzers</t>
-        </is>
-      </c>
-      <c r="D35" s="87" t="inlineStr">
-        <is>
-          <t>Low-A</t>
-        </is>
-      </c>
-      <c r="E35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N35" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O35" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="86" t="inlineStr">
-        <is>
-          <t>Evan Chrest</t>
-        </is>
-      </c>
-      <c r="B36" s="86" t="inlineStr">
-        <is>
-          <t>RHP</t>
-        </is>
-      </c>
-      <c r="C36" s="87" t="inlineStr">
-        <is>
-          <t>ACL/AZL</t>
-        </is>
-      </c>
-      <c r="D36" s="87" t="inlineStr">
-        <is>
-          <t>Rookie</t>
-        </is>
-      </c>
-      <c r="E36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N36" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O36" s="87" t="inlineStr">
-        <is>
-          <t>04/24/2026 20:04</t>
+          <t>04/24/2026 20:07</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A14:O14"/>
+    <mergeCell ref="A4:O4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove Jack Anderson news card; add Cole Sands to 15-Day IL; add 15-Day IL support
</commit_message>
<xml_diff>
--- a/noles_in_the_pros.xlsx
+++ b/noles_in_the_pros.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6" yWindow="6" windowWidth="23028" windowHeight="13668" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$K$35</definedName>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>15-Day IL</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -1140,6 +1140,11 @@
       <c r="K6" s="5" t="inlineStr">
         <is>
           <t>69 G, 72 IP, 4.50 ERA in 2025; re-signed 1yr/$1.1M</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>MLB</t>
         </is>
       </c>
     </row>

</xml_diff>